<commit_message>
account creation kyc updation
</commit_message>
<xml_diff>
--- a/kalarakal_updated.xlsx
+++ b/kalarakal_updated.xlsx
@@ -3,14 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chella\eclipse-workspace\mavenCrm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32532346-17E1-4884-A79F-CFA71C0908EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CA589EE-A1E7-409F-9607-67D279055D22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="971" uniqueCount="534">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="975" uniqueCount="531">
   <si>
     <t>Status</t>
   </si>
@@ -1582,12 +1582,6 @@
     <t>panNo</t>
   </si>
   <si>
-    <t>4 Pass 1 Fail</t>
-  </si>
-  <si>
-    <t>62 Sec</t>
-  </si>
-  <si>
     <t>panFront</t>
   </si>
   <si>
@@ -1600,9 +1594,6 @@
     <t>pan_02</t>
   </si>
   <si>
-    <t>Digi Gold</t>
-  </si>
-  <si>
     <t>aadharFront</t>
   </si>
   <si>
@@ -1621,24 +1612,23 @@
     <t>XYZPC9999K</t>
   </si>
   <si>
-    <t>11 Sec</t>
-  </si>
-  <si>
     <t>DG-not allocated</t>
   </si>
   <si>
-    <t>10 Sec</t>
-  </si>
-  <si>
-    <t>24 Sec</t>
+    <t>Digi silver</t>
+  </si>
+  <si>
+    <t>36 Sec</t>
+  </si>
+  <si>
+    <t>14 Sec</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
-  <fonts count="33" x14ac:knownFonts="1">
+  <fonts count="30" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1807,7 +1797,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color indexed="17"/>
+      <color indexed="10"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -1821,24 +1811,6 @@
       <sz val="11"/>
       <color indexed="10"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-      <color indexed="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-      <color indexed="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-      <color indexed="10"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1862,7 +1834,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
@@ -1894,13 +1866,10 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="true"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2185,124 +2154,127 @@
   <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="12.7265625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="7.81640625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="13.90625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="5.0"/>
+    <col min="1" max="1" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>21</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" t="s" s="0">
+      <c r="A2" t="s">
         <v>23</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>12</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="C2" t="s">
         <v>510</v>
       </c>
-      <c r="D2" t="s" s="0">
-        <v>533</v>
+      <c r="D2" t="s">
+        <v>530</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" t="s" s="0">
+      <c r="A3" t="s">
         <v>2</v>
       </c>
-      <c r="B3" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="C3" t="s" s="0">
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
         <v>495</v>
       </c>
-      <c r="D3" t="s" s="0">
+      <c r="D3" t="s">
         <v>511</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4" t="s" s="0">
+      <c r="A4" t="s">
         <v>34</v>
       </c>
-      <c r="B4" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="C4" t="s" s="0">
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
         <v>495</v>
       </c>
-      <c r="D4" t="s" s="0">
+      <c r="D4" t="s">
         <v>497</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A5" t="s" s="0">
+      <c r="A5" t="s">
         <v>24</v>
       </c>
-      <c r="B5" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="C5" t="s" s="0">
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
         <v>495</v>
       </c>
-      <c r="D5" t="s" s="0">
+      <c r="D5" t="s">
         <v>514</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A6" t="s" s="0">
+      <c r="A6" t="s">
         <v>25</v>
       </c>
-      <c r="B6" t="s" s="0">
-        <v>9</v>
+      <c r="B6" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A7" t="s" s="0">
+      <c r="A7" t="s">
         <v>26</v>
       </c>
-      <c r="B7" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="C7" t="s" s="0">
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" t="s">
         <v>499</v>
       </c>
-      <c r="D7" t="s" s="0">
+      <c r="D7" t="s">
         <v>512</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A8" t="s" s="0">
+      <c r="A8" t="s">
         <v>27</v>
       </c>
-      <c r="C8" t="s" s="0">
-        <v>517</v>
-      </c>
-      <c r="D8" t="s" s="0">
-        <v>518</v>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="s">
+        <v>510</v>
+      </c>
+      <c r="D8" t="s">
+        <v>529</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A9" t="s" s="0">
+      <c r="A9" t="s">
         <v>28</v>
       </c>
-      <c r="B9" t="s" s="0">
-        <v>12</v>
-      </c>
-      <c r="C9" t="s" s="0">
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" t="s">
         <v>510</v>
       </c>
-      <c r="D9" t="s" s="0">
-        <v>527</v>
+      <c r="D9" t="s">
+        <v>524</v>
       </c>
     </row>
   </sheetData>
@@ -2319,25 +2291,25 @@
       <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>14</v>
       </c>
-      <c r="C3" t="s" s="0">
+      <c r="C3" t="s">
         <v>490</v>
       </c>
-      <c r="E3" t="s" s="0">
+      <c r="E3" t="s">
         <v>508</v>
       </c>
-      <c r="H3" t="s" s="0">
+      <c r="H3" t="s">
         <v>509</v>
       </c>
-      <c r="I3" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="N3" t="s" s="0">
+      <c r="I3" t="s">
+        <v>9</v>
+      </c>
+      <c r="N3" t="s">
         <v>461</v>
       </c>
-      <c r="O3" s="0">
+      <c r="O3">
         <v>0</v>
       </c>
     </row>
@@ -2351,44 +2323,44 @@
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="5.90625"/>
-    <col min="2" max="2" customWidth="true" width="5.90625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="9.1796875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="62.0"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="16.0"/>
+    <col min="1" max="1" width="5.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.90625" customWidth="1"/>
+    <col min="3" max="3" width="9.1796875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="62" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>29</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>30</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="32" t="s">
         <v>513</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="C2" t="s">
         <v>32</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>493</v>
       </c>
-      <c r="E2" t="s" s="0">
+      <c r="E2" t="s">
         <v>33</v>
       </c>
     </row>
@@ -2405,29 +2377,29 @@
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" customWidth="true" width="10.0"/>
-    <col min="3" max="3" customWidth="true" width="22.0"/>
-    <col min="4" max="5" customWidth="true" width="8.0"/>
-    <col min="6" max="6" customWidth="true" width="25.0"/>
+    <col min="1" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="5" width="8" customWidth="1"/>
+    <col min="6" max="6" width="25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -2435,16 +2407,16 @@
       <c r="A2" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="C2" t="s">
         <v>8</v>
       </c>
-      <c r="D2" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="E2" t="s" s="0">
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -2452,19 +2424,19 @@
       <c r="A3" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" t="s" s="0">
+      <c r="C3" t="s">
         <v>11</v>
       </c>
-      <c r="D3" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="F3" t="s" s="0">
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" t="s">
         <v>13</v>
       </c>
     </row>
@@ -2472,16 +2444,16 @@
       <c r="A4" s="15" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="B4" t="s">
         <v>14</v>
       </c>
-      <c r="C4" t="s" s="0">
+      <c r="C4" t="s">
         <v>15</v>
       </c>
-      <c r="D4" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="E4" t="s" s="0">
+      <c r="D4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" t="s">
         <v>9</v>
       </c>
     </row>
@@ -2489,19 +2461,19 @@
       <c r="A5" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B5" t="s" s="0">
+      <c r="B5" t="s">
         <v>16</v>
       </c>
-      <c r="C5" t="s" s="0">
+      <c r="C5" t="s">
         <v>17</v>
       </c>
-      <c r="D5" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="E5" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="F5" t="s" s="0">
+      <c r="D5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" t="s">
         <v>494</v>
       </c>
     </row>
@@ -2509,16 +2481,16 @@
       <c r="A6" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="B6" t="s" s="0">
+      <c r="B6" t="s">
         <v>18</v>
       </c>
-      <c r="C6" t="s" s="0">
+      <c r="C6" t="s">
         <v>19</v>
       </c>
-      <c r="D6" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="E6" t="s" s="0">
+      <c r="D6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" t="s">
         <v>9</v>
       </c>
     </row>
@@ -2532,29 +2504,29 @@
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" customWidth="true" width="10.0"/>
-    <col min="3" max="3" customWidth="true" width="22.0"/>
-    <col min="4" max="5" customWidth="true" width="8.0"/>
-    <col min="6" max="6" customWidth="true" width="25.0"/>
+    <col min="1" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="5" width="8" customWidth="1"/>
+    <col min="6" max="6" width="25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>34</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s">
         <v>35</v>
       </c>
     </row>
@@ -2562,16 +2534,16 @@
       <c r="A2" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="C2" t="s">
         <v>36</v>
       </c>
-      <c r="D2" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="E2" t="s" s="0">
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -2579,19 +2551,19 @@
       <c r="A3" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" t="s" s="0">
+      <c r="C3" t="s">
         <v>37</v>
       </c>
-      <c r="D3" t="s" s="0">
+      <c r="D3" t="s">
         <v>12</v>
       </c>
-      <c r="E3" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="F3" t="s" s="0">
+      <c r="E3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" t="s">
         <v>38</v>
       </c>
     </row>
@@ -2599,16 +2571,16 @@
       <c r="A4" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="B4" t="s">
         <v>14</v>
       </c>
-      <c r="C4" t="s" s="0">
+      <c r="C4" t="s">
         <v>39</v>
       </c>
-      <c r="D4" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="E4" t="s" s="0">
+      <c r="D4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" t="s">
         <v>9</v>
       </c>
     </row>
@@ -2616,19 +2588,19 @@
       <c r="A5" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B5" t="s" s="0">
+      <c r="B5" t="s">
         <v>16</v>
       </c>
-      <c r="C5" t="s" s="0">
+      <c r="C5" t="s">
         <v>40</v>
       </c>
-      <c r="D5" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="E5" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="F5" t="s" s="0">
+      <c r="D5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" t="s">
         <v>41</v>
       </c>
     </row>
@@ -2636,16 +2608,16 @@
       <c r="A6" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="B6" t="s" s="0">
+      <c r="B6" t="s">
         <v>18</v>
       </c>
-      <c r="C6" t="s" s="0">
+      <c r="C6" t="s">
         <v>42</v>
       </c>
-      <c r="D6" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="E6" t="s" s="0">
+      <c r="D6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" t="s">
         <v>9</v>
       </c>
     </row>
@@ -2659,29 +2631,29 @@
   <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" customWidth="true" width="10.0"/>
-    <col min="3" max="3" customWidth="true" width="22.0"/>
-    <col min="4" max="5" customWidth="true" width="8.0"/>
-    <col min="6" max="6" customWidth="true" width="25.0"/>
+    <col min="1" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="5" width="8" customWidth="1"/>
+    <col min="6" max="6" width="25" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>24</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s">
         <v>43</v>
       </c>
     </row>
@@ -2689,16 +2661,16 @@
       <c r="A2" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="C2" t="s">
         <v>44</v>
       </c>
-      <c r="D2" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="E2" t="s" s="0">
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -2706,19 +2678,19 @@
       <c r="A3" s="24" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" t="s" s="0">
+      <c r="C3" t="s">
         <v>45</v>
       </c>
-      <c r="D3" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="E3" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="F3" t="s" s="0">
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" t="s">
+        <v>9</v>
+      </c>
+      <c r="F3" t="s">
         <v>46</v>
       </c>
     </row>
@@ -2726,16 +2698,16 @@
       <c r="A4" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="B4" t="s">
         <v>14</v>
       </c>
-      <c r="C4" t="s" s="0">
+      <c r="C4" t="s">
         <v>47</v>
       </c>
-      <c r="D4" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="E4" t="s" s="0">
+      <c r="D4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" t="s">
         <v>9</v>
       </c>
     </row>
@@ -2743,19 +2715,19 @@
       <c r="A5" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="B5" t="s" s="0">
+      <c r="B5" t="s">
         <v>16</v>
       </c>
-      <c r="C5" t="s" s="0">
+      <c r="C5" t="s">
         <v>48</v>
       </c>
-      <c r="D5" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="E5" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="F5" t="s" s="0">
+      <c r="D5" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" t="s">
         <v>49</v>
       </c>
     </row>
@@ -2763,13 +2735,13 @@
       <c r="A6" s="27" t="s">
         <v>6</v>
       </c>
-      <c r="B6" t="s" s="0">
+      <c r="B6" t="s">
         <v>18</v>
       </c>
-      <c r="D6" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="E6" t="s" s="0">
+      <c r="D6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" t="s">
         <v>9</v>
       </c>
     </row>
@@ -2783,284 +2755,284 @@
   <dimension ref="A1:BR10"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" bestFit="true" customWidth="true" width="5.90625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="12.6328125"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="4.36328125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="16.6328125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="9.0"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="8.6328125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="10.81640625"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="9.54296875"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="20.90625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="7.453125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="22.90625"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="12.453125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="19.90625"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="18.08984375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="11.26953125"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="7.453125"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="10.26953125"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="10.6328125"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="7.36328125"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="14.453125"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="12.08984375"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="7.0"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="10.54296875"/>
-    <col min="26" max="27" bestFit="true" customWidth="true" width="11.81640625"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" width="8.81640625"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="13.6328125"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="15.54296875"/>
-    <col min="31" max="31" bestFit="true" customWidth="true" width="15.08984375"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" width="17.36328125"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" width="12.54296875"/>
-    <col min="34" max="34" bestFit="true" customWidth="true" width="10.36328125"/>
-    <col min="35" max="36" bestFit="true" customWidth="true" width="12.0"/>
-    <col min="37" max="37" bestFit="true" customWidth="true" width="12.7265625"/>
-    <col min="38" max="38" bestFit="true" customWidth="true" width="3.6328125"/>
-    <col min="39" max="39" bestFit="true" customWidth="true" width="4.90625"/>
-    <col min="40" max="40" bestFit="true" customWidth="true" width="16.453125"/>
-    <col min="41" max="41" bestFit="true" customWidth="true" width="19.0"/>
-    <col min="42" max="42" bestFit="true" customWidth="true" width="14.90625"/>
-    <col min="43" max="43" bestFit="true" customWidth="true" width="12.36328125"/>
-    <col min="44" max="44" bestFit="true" customWidth="true" width="17.08984375"/>
-    <col min="45" max="45" bestFit="true" customWidth="true" width="10.54296875"/>
-    <col min="46" max="46" bestFit="true" customWidth="true" width="13.90625"/>
-    <col min="47" max="47" bestFit="true" customWidth="true" width="7.90625"/>
-    <col min="48" max="48" bestFit="true" customWidth="true" width="12.0"/>
-    <col min="49" max="49" bestFit="true" customWidth="true" width="9.54296875"/>
-    <col min="50" max="50" bestFit="true" customWidth="true" width="10.81640625"/>
-    <col min="51" max="51" bestFit="true" customWidth="true" width="13.36328125"/>
-    <col min="52" max="52" bestFit="true" customWidth="true" width="6.90625"/>
-    <col min="53" max="53" bestFit="true" customWidth="true" width="12.90625"/>
-    <col min="54" max="54" bestFit="true" customWidth="true" width="10.54296875"/>
-    <col min="55" max="55" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="56" max="56" bestFit="true" customWidth="true" width="14.1796875"/>
-    <col min="57" max="57" bestFit="true" customWidth="true" width="13.36328125"/>
-    <col min="58" max="58" bestFit="true" customWidth="true" width="9.08984375"/>
-    <col min="59" max="59" bestFit="true" customWidth="true" width="16.1796875"/>
-    <col min="60" max="60" bestFit="true" customWidth="true" width="8.08984375"/>
-    <col min="61" max="61" bestFit="true" customWidth="true" width="10.453125"/>
-    <col min="62" max="62" bestFit="true" customWidth="true" width="14.26953125"/>
-    <col min="63" max="63" bestFit="true" customWidth="true" width="11.26953125"/>
-    <col min="64" max="64" bestFit="true" customWidth="true" width="4.0"/>
-    <col min="65" max="65" bestFit="true" customWidth="true" width="6.0"/>
-    <col min="66" max="66" bestFit="true" customWidth="true" width="12.36328125"/>
-    <col min="67" max="67" bestFit="true" customWidth="true" width="10.81640625"/>
-    <col min="68" max="68" bestFit="true" customWidth="true" width="25.36328125"/>
-    <col min="69" max="69" bestFit="true" customWidth="true" width="22.6328125"/>
-    <col min="70" max="70" bestFit="true" customWidth="true" width="15.6328125"/>
+    <col min="1" max="2" width="5.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.36328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.90625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="22.90625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.90625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.08984375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="7.36328125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.453125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="7" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="26" max="27" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="13.6328125" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="17.36328125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="12" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="3.6328125" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="4.90625" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="16.453125" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="19" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="14.90625" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="7.90625" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="12" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="9.54296875" bestFit="1" customWidth="1"/>
+    <col min="50" max="50" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="51" max="51" width="13.36328125" bestFit="1" customWidth="1"/>
+    <col min="52" max="52" width="6.90625" bestFit="1" customWidth="1"/>
+    <col min="53" max="53" width="12.90625" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="55" max="55" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="56" max="56" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="57" max="57" width="13.36328125" bestFit="1" customWidth="1"/>
+    <col min="58" max="58" width="9.08984375" bestFit="1" customWidth="1"/>
+    <col min="59" max="59" width="16.1796875" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="8.08984375" bestFit="1" customWidth="1"/>
+    <col min="61" max="61" width="10.453125" bestFit="1" customWidth="1"/>
+    <col min="62" max="62" width="14.26953125" bestFit="1" customWidth="1"/>
+    <col min="63" max="63" width="11.26953125" bestFit="1" customWidth="1"/>
+    <col min="64" max="64" width="4" bestFit="1" customWidth="1"/>
+    <col min="65" max="65" width="6" bestFit="1" customWidth="1"/>
+    <col min="66" max="66" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="67" max="67" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="68" max="68" width="25.36328125" bestFit="1" customWidth="1"/>
+    <col min="69" max="69" width="22.6328125" bestFit="1" customWidth="1"/>
+    <col min="70" max="70" width="15.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:70" x14ac:dyDescent="0.35">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>51</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>52</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>53</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s">
         <v>54</v>
       </c>
-      <c r="G1" t="s" s="0">
+      <c r="G1" t="s">
         <v>55</v>
       </c>
-      <c r="H1" t="s" s="0">
+      <c r="H1" t="s">
         <v>56</v>
       </c>
-      <c r="I1" t="s" s="0">
+      <c r="I1" t="s">
         <v>57</v>
       </c>
-      <c r="J1" t="s" s="0">
+      <c r="J1" t="s">
         <v>24</v>
       </c>
-      <c r="K1" t="s" s="0">
+      <c r="K1" t="s">
         <v>58</v>
       </c>
-      <c r="L1" t="s" s="0">
+      <c r="L1" t="s">
         <v>59</v>
       </c>
-      <c r="M1" t="s" s="0">
+      <c r="M1" t="s">
         <v>60</v>
       </c>
-      <c r="N1" t="s" s="0">
+      <c r="N1" t="s">
         <v>61</v>
       </c>
-      <c r="O1" t="s" s="0">
+      <c r="O1" t="s">
         <v>62</v>
       </c>
-      <c r="P1" t="s" s="0">
+      <c r="P1" t="s">
         <v>63</v>
       </c>
-      <c r="Q1" t="s" s="0">
+      <c r="Q1" t="s">
         <v>64</v>
       </c>
-      <c r="R1" t="s" s="0">
+      <c r="R1" t="s">
         <v>65</v>
       </c>
-      <c r="S1" t="s" s="0">
+      <c r="S1" t="s">
         <v>66</v>
       </c>
-      <c r="T1" t="s" s="0">
+      <c r="T1" t="s">
         <v>67</v>
       </c>
-      <c r="U1" t="s" s="0">
+      <c r="U1" t="s">
         <v>68</v>
       </c>
-      <c r="V1" t="s" s="0">
+      <c r="V1" t="s">
         <v>69</v>
       </c>
-      <c r="W1" t="s" s="0">
+      <c r="W1" t="s">
         <v>70</v>
       </c>
-      <c r="X1" t="s" s="0">
+      <c r="X1" t="s">
         <v>71</v>
       </c>
-      <c r="Y1" t="s" s="0">
+      <c r="Y1" t="s">
         <v>72</v>
       </c>
-      <c r="Z1" t="s" s="0">
+      <c r="Z1" t="s">
         <v>73</v>
       </c>
-      <c r="AA1" t="s" s="0">
+      <c r="AA1" t="s">
         <v>74</v>
       </c>
-      <c r="AB1" t="s" s="0">
+      <c r="AB1" t="s">
         <v>75</v>
       </c>
-      <c r="AC1" t="s" s="0">
+      <c r="AC1" t="s">
         <v>76</v>
       </c>
-      <c r="AD1" t="s" s="0">
+      <c r="AD1" t="s">
         <v>77</v>
       </c>
-      <c r="AE1" t="s" s="0">
+      <c r="AE1" t="s">
         <v>78</v>
       </c>
-      <c r="AF1" t="s" s="0">
+      <c r="AF1" t="s">
         <v>79</v>
       </c>
-      <c r="AG1" t="s" s="0">
+      <c r="AG1" t="s">
         <v>80</v>
       </c>
-      <c r="AH1" t="s" s="0">
+      <c r="AH1" t="s">
         <v>81</v>
       </c>
-      <c r="AI1" t="s" s="0">
+      <c r="AI1" t="s">
         <v>82</v>
       </c>
-      <c r="AJ1" t="s" s="0">
+      <c r="AJ1" t="s">
         <v>83</v>
       </c>
-      <c r="AK1" t="s" s="0">
+      <c r="AK1" t="s">
         <v>84</v>
       </c>
-      <c r="AL1" t="s" s="0">
+      <c r="AL1" t="s">
         <v>85</v>
       </c>
-      <c r="AM1" t="s" s="0">
+      <c r="AM1" t="s">
         <v>86</v>
       </c>
-      <c r="AN1" t="s" s="0">
+      <c r="AN1" t="s">
         <v>87</v>
       </c>
-      <c r="AO1" t="s" s="0">
+      <c r="AO1" t="s">
         <v>88</v>
       </c>
-      <c r="AP1" t="s" s="0">
+      <c r="AP1" t="s">
         <v>89</v>
       </c>
-      <c r="AQ1" t="s" s="0">
+      <c r="AQ1" t="s">
         <v>90</v>
       </c>
-      <c r="AR1" t="s" s="0">
+      <c r="AR1" t="s">
         <v>91</v>
       </c>
-      <c r="AS1" t="s" s="0">
+      <c r="AS1" t="s">
         <v>92</v>
       </c>
-      <c r="AT1" t="s" s="0">
+      <c r="AT1" t="s">
         <v>93</v>
       </c>
-      <c r="AU1" t="s" s="0">
+      <c r="AU1" t="s">
         <v>94</v>
       </c>
-      <c r="AV1" t="s" s="0">
+      <c r="AV1" t="s">
         <v>95</v>
       </c>
-      <c r="AW1" t="s" s="0">
+      <c r="AW1" t="s">
         <v>96</v>
       </c>
-      <c r="AX1" t="s" s="0">
+      <c r="AX1" t="s">
         <v>97</v>
       </c>
-      <c r="AY1" t="s" s="0">
+      <c r="AY1" t="s">
         <v>98</v>
       </c>
-      <c r="AZ1" t="s" s="0">
+      <c r="AZ1" t="s">
         <v>99</v>
       </c>
-      <c r="BA1" t="s" s="0">
+      <c r="BA1" t="s">
         <v>100</v>
       </c>
-      <c r="BB1" t="s" s="0">
+      <c r="BB1" t="s">
         <v>101</v>
       </c>
-      <c r="BC1" t="s" s="0">
+      <c r="BC1" t="s">
         <v>102</v>
       </c>
-      <c r="BD1" t="s" s="0">
+      <c r="BD1" t="s">
         <v>103</v>
       </c>
-      <c r="BE1" t="s" s="0">
+      <c r="BE1" t="s">
         <v>104</v>
       </c>
-      <c r="BF1" t="s" s="0">
+      <c r="BF1" t="s">
         <v>105</v>
       </c>
-      <c r="BG1" t="s" s="0">
+      <c r="BG1" t="s">
         <v>106</v>
       </c>
-      <c r="BH1" t="s" s="0">
+      <c r="BH1" t="s">
         <v>107</v>
       </c>
-      <c r="BI1" t="s" s="0">
+      <c r="BI1" t="s">
         <v>108</v>
       </c>
-      <c r="BJ1" t="s" s="0">
+      <c r="BJ1" t="s">
         <v>109</v>
       </c>
-      <c r="BK1" t="s" s="0">
+      <c r="BK1" t="s">
         <v>110</v>
       </c>
-      <c r="BL1" t="s" s="0">
+      <c r="BL1" t="s">
         <v>3</v>
       </c>
-      <c r="BM1" t="s" s="0">
+      <c r="BM1" t="s">
         <v>4</v>
       </c>
-      <c r="BN1" t="s" s="0">
+      <c r="BN1" t="s">
         <v>111</v>
       </c>
-      <c r="BO1" t="s" s="0">
+      <c r="BO1" t="s">
         <v>112</v>
       </c>
-      <c r="BP1" t="s" s="0">
+      <c r="BP1" t="s">
         <v>113</v>
       </c>
-      <c r="BQ1" t="s" s="0">
+      <c r="BQ1" t="s">
         <v>114</v>
       </c>
-      <c r="BR1" t="s" s="0">
+      <c r="BR1" t="s">
         <v>115</v>
       </c>
     </row>
@@ -4467,137 +4439,137 @@
   <dimension ref="A1:AG9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" bestFit="true" customWidth="true" width="5.90625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="9.0"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="8.6328125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="8.81640625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="3.6328125"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="13.36328125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="10.90625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="5.81640625"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="17.08984375"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="14.7265625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="10.6328125"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="7.7265625"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="7.453125"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="10.26953125"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="10.6328125"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="12.453125"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="10.81640625"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="26.90625"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="13.08984375"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="12.36328125"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="11.08984375"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="20.1796875"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="12.08984375"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="4.0"/>
-    <col min="26" max="27" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" width="12.0"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="14.1796875"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="16.08984375"/>
-    <col min="31" max="31" bestFit="true" customWidth="true" width="12.7265625"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" width="14.0"/>
-    <col min="33" max="33" bestFit="true" customWidth="true" width="6.0"/>
+    <col min="1" max="2" width="5.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.6328125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="3.6328125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="5.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.7265625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="7.453125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="12.453125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="26.90625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="13.08984375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="12.36328125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="11.08984375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="20.1796875" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="4" bestFit="1" customWidth="1"/>
+    <col min="26" max="27" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="12" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="14.1796875" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="14" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="6" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:33" x14ac:dyDescent="0.35">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>353</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s">
         <v>354</v>
       </c>
-      <c r="G1" t="s" s="0">
+      <c r="G1" t="s">
         <v>34</v>
       </c>
-      <c r="H1" t="s" s="0">
+      <c r="H1" t="s">
         <v>2</v>
       </c>
-      <c r="I1" t="s" s="0">
+      <c r="I1" t="s">
         <v>355</v>
       </c>
-      <c r="J1" t="s" s="0">
+      <c r="J1" t="s">
         <v>356</v>
       </c>
-      <c r="K1" t="s" s="0">
+      <c r="K1" t="s">
         <v>357</v>
       </c>
-      <c r="L1" t="s" s="0">
+      <c r="L1" t="s">
         <v>358</v>
       </c>
-      <c r="M1" t="s" s="0">
+      <c r="M1" t="s">
         <v>359</v>
       </c>
-      <c r="N1" t="s" s="0">
+      <c r="N1" t="s">
         <v>65</v>
       </c>
-      <c r="O1" t="s" s="0">
+      <c r="O1" t="s">
         <v>66</v>
       </c>
-      <c r="P1" t="s" s="0">
+      <c r="P1" t="s">
         <v>67</v>
       </c>
-      <c r="Q1" t="s" s="0">
+      <c r="Q1" t="s">
         <v>61</v>
       </c>
-      <c r="R1" t="s" s="0">
+      <c r="R1" t="s">
         <v>57</v>
       </c>
-      <c r="S1" t="s" s="0">
+      <c r="S1" t="s">
         <v>360</v>
       </c>
-      <c r="T1" t="s" s="0">
+      <c r="T1" t="s">
         <v>361</v>
       </c>
-      <c r="U1" t="s" s="0">
+      <c r="U1" t="s">
         <v>110</v>
       </c>
-      <c r="V1" t="s" s="0">
+      <c r="V1" t="s">
         <v>362</v>
       </c>
-      <c r="W1" t="s" s="0">
+      <c r="W1" t="s">
         <v>363</v>
       </c>
-      <c r="X1" t="s" s="0">
+      <c r="X1" t="s">
         <v>364</v>
       </c>
-      <c r="Y1" t="s" s="0">
+      <c r="Y1" t="s">
         <v>3</v>
       </c>
-      <c r="Z1" t="s" s="0">
+      <c r="Z1" t="s">
         <v>365</v>
       </c>
-      <c r="AA1" t="s" s="0">
+      <c r="AA1" t="s">
         <v>366</v>
       </c>
-      <c r="AB1" t="s" s="0">
+      <c r="AB1" t="s">
         <v>367</v>
       </c>
-      <c r="AC1" t="s" s="0">
+      <c r="AC1" t="s">
         <v>5</v>
       </c>
-      <c r="AD1" t="s" s="0">
+      <c r="AD1" t="s">
         <v>35</v>
       </c>
-      <c r="AE1" t="s" s="0">
+      <c r="AE1" t="s">
         <v>368</v>
       </c>
-      <c r="AF1" t="s" s="0">
+      <c r="AF1" t="s">
         <v>369</v>
       </c>
-      <c r="AG1" t="s" s="0">
+      <c r="AG1" t="s">
         <v>4</v>
       </c>
     </row>
@@ -4605,97 +4577,97 @@
       <c r="A2" s="28" t="s">
         <v>513</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="C2" t="s">
         <v>370</v>
       </c>
-      <c r="D2" t="s" s="0">
+      <c r="D2" t="s">
         <v>119</v>
       </c>
-      <c r="E2" t="s" s="0">
+      <c r="E2" t="s">
         <v>371</v>
       </c>
-      <c r="G2" t="s" s="0">
+      <c r="G2" t="s">
         <v>36</v>
       </c>
-      <c r="H2" t="s" s="0">
+      <c r="H2" t="s">
         <v>8</v>
       </c>
-      <c r="I2" t="s" s="0">
+      <c r="I2" t="s">
         <v>12</v>
       </c>
-      <c r="J2" t="s" s="0">
+      <c r="J2" t="s">
         <v>372</v>
       </c>
-      <c r="K2" t="s" s="0">
+      <c r="K2" t="s">
         <v>373</v>
       </c>
-      <c r="L2" t="s" s="0">
+      <c r="L2" t="s">
         <v>300</v>
       </c>
-      <c r="M2" t="s" s="0">
+      <c r="M2" t="s">
         <v>301</v>
       </c>
-      <c r="N2" t="s" s="0">
+      <c r="N2" t="s">
         <v>128</v>
       </c>
-      <c r="O2" t="s" s="0">
+      <c r="O2" t="s">
         <v>129</v>
       </c>
-      <c r="P2" t="s" s="0">
+      <c r="P2" t="s">
         <v>300</v>
       </c>
-      <c r="Q2" t="s" s="0">
+      <c r="Q2" t="s">
         <v>374</v>
       </c>
-      <c r="R2" t="s" s="0">
+      <c r="R2" t="s">
         <v>120</v>
       </c>
-      <c r="S2" t="s" s="0">
+      <c r="S2" t="s">
         <v>375</v>
       </c>
-      <c r="T2" t="s" s="0">
+      <c r="T2" t="s">
         <v>376</v>
       </c>
-      <c r="U2" t="s" s="0">
+      <c r="U2" t="s">
         <v>377</v>
       </c>
-      <c r="V2" t="s" s="0">
+      <c r="V2" t="s">
         <v>492</v>
       </c>
-      <c r="W2" t="s" s="0">
+      <c r="W2" t="s">
         <v>490</v>
       </c>
-      <c r="X2" t="s" s="0">
+      <c r="X2" t="s">
         <v>378</v>
       </c>
-      <c r="Y2" t="s" s="0">
+      <c r="Y2" t="s">
         <v>12</v>
       </c>
-      <c r="Z2" t="s" s="0">
+      <c r="Z2" t="s">
         <v>379</v>
       </c>
-      <c r="AA2" t="s" s="0">
+      <c r="AA2" t="s">
         <v>322</v>
       </c>
-      <c r="AB2" t="s" s="0">
+      <c r="AB2" t="s">
         <v>380</v>
       </c>
-      <c r="AC2" t="s" s="0">
+      <c r="AC2" t="s">
         <v>381</v>
       </c>
-      <c r="AD2" t="s" s="0">
+      <c r="AD2" t="s">
         <v>40</v>
       </c>
-      <c r="AE2" t="s" s="0">
+      <c r="AE2" t="s">
         <v>382</v>
       </c>
-      <c r="AF2" t="s" s="0">
+      <c r="AF2" t="s">
         <v>383</v>
       </c>
-      <c r="AG2" t="s" s="0">
+      <c r="AG2" t="s">
         <v>9</v>
       </c>
     </row>
@@ -4703,76 +4675,76 @@
       <c r="A3" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B3" t="s" s="0">
+      <c r="B3" t="s">
         <v>10</v>
       </c>
-      <c r="C3" t="s" s="0">
+      <c r="C3" t="s">
         <v>249</v>
       </c>
-      <c r="D3" t="s" s="0">
+      <c r="D3" t="s">
         <v>250</v>
       </c>
-      <c r="E3" t="s" s="0">
+      <c r="E3" t="s">
         <v>384</v>
       </c>
-      <c r="G3" t="s" s="0">
+      <c r="G3" t="s">
         <v>496</v>
       </c>
-      <c r="H3" t="s" s="0">
+      <c r="H3" t="s">
         <v>11</v>
       </c>
-      <c r="I3" t="s" s="0">
+      <c r="I3" t="s">
         <v>12</v>
       </c>
-      <c r="J3" t="s" s="0">
+      <c r="J3" t="s">
         <v>167</v>
       </c>
-      <c r="K3" t="s" s="0">
+      <c r="K3" t="s">
         <v>168</v>
       </c>
-      <c r="L3" t="s" s="0">
+      <c r="L3" t="s">
         <v>169</v>
       </c>
-      <c r="M3" t="s" s="0">
+      <c r="M3" t="s">
         <v>170</v>
       </c>
-      <c r="N3" t="s" s="0">
+      <c r="N3" t="s">
         <v>128</v>
       </c>
-      <c r="O3" t="s" s="0">
+      <c r="O3" t="s">
         <v>129</v>
       </c>
-      <c r="P3" t="s" s="0">
+      <c r="P3" t="s">
         <v>169</v>
       </c>
-      <c r="Q3" t="s" s="0">
+      <c r="Q3" t="s">
         <v>385</v>
       </c>
-      <c r="R3" t="s" s="0">
+      <c r="R3" t="s">
         <v>163</v>
       </c>
-      <c r="S3" t="s" s="0">
+      <c r="S3" t="s">
         <v>386</v>
       </c>
-      <c r="T3" t="s" s="0">
+      <c r="T3" t="s">
         <v>387</v>
       </c>
-      <c r="U3" t="s" s="0">
+      <c r="U3" t="s">
         <v>388</v>
       </c>
-      <c r="V3" t="s" s="0">
+      <c r="V3" t="s">
         <v>492</v>
       </c>
-      <c r="W3" t="s" s="0">
+      <c r="W3" t="s">
         <v>491</v>
       </c>
-      <c r="X3" t="s" s="0">
+      <c r="X3" t="s">
         <v>389</v>
       </c>
-      <c r="Y3" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="AG3" t="s" s="0">
+      <c r="Y3" t="s">
+        <v>9</v>
+      </c>
+      <c r="AG3" t="s">
         <v>9</v>
       </c>
     </row>
@@ -4780,76 +4752,76 @@
       <c r="A4" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s" s="0">
+      <c r="B4" t="s">
         <v>14</v>
       </c>
-      <c r="C4" t="s" s="0">
+      <c r="C4" t="s">
         <v>209</v>
       </c>
-      <c r="D4" t="s" s="0">
+      <c r="D4" t="s">
         <v>210</v>
       </c>
-      <c r="E4" t="s" s="0">
+      <c r="E4" t="s">
         <v>390</v>
       </c>
-      <c r="G4" t="s" s="0">
+      <c r="G4" t="s">
         <v>39</v>
       </c>
-      <c r="H4" t="s" s="0">
+      <c r="H4" t="s">
         <v>15</v>
       </c>
-      <c r="I4" t="s" s="0">
+      <c r="I4" t="s">
         <v>12</v>
       </c>
-      <c r="J4" t="s" s="0">
+      <c r="J4" t="s">
         <v>391</v>
       </c>
-      <c r="K4" t="s" s="0">
+      <c r="K4" t="s">
         <v>392</v>
       </c>
-      <c r="L4" t="s" s="0">
+      <c r="L4" t="s">
         <v>258</v>
       </c>
-      <c r="M4" t="s" s="0">
+      <c r="M4" t="s">
         <v>259</v>
       </c>
-      <c r="N4" t="s" s="0">
+      <c r="N4" t="s">
         <v>128</v>
       </c>
-      <c r="O4" t="s" s="0">
+      <c r="O4" t="s">
         <v>129</v>
       </c>
-      <c r="P4" t="s" s="0">
+      <c r="P4" t="s">
         <v>258</v>
       </c>
-      <c r="Q4" t="s" s="0">
+      <c r="Q4" t="s">
         <v>393</v>
       </c>
-      <c r="R4" t="s" s="0">
+      <c r="R4" t="s">
         <v>184</v>
       </c>
-      <c r="S4" t="s" s="0">
+      <c r="S4" t="s">
         <v>394</v>
       </c>
-      <c r="T4" t="s" s="0">
+      <c r="T4" t="s">
         <v>395</v>
       </c>
-      <c r="U4" t="s" s="0">
+      <c r="U4" t="s">
         <v>396</v>
       </c>
-      <c r="V4" t="s" s="0">
+      <c r="V4" t="s">
         <v>492</v>
       </c>
-      <c r="W4" t="s" s="0">
+      <c r="W4" t="s">
         <v>491</v>
       </c>
-      <c r="X4" t="s" s="0">
+      <c r="X4" t="s">
         <v>397</v>
       </c>
-      <c r="Y4" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="AG4" t="s" s="0">
+      <c r="Y4" t="s">
+        <v>9</v>
+      </c>
+      <c r="AG4" t="s">
         <v>9</v>
       </c>
     </row>
@@ -4857,97 +4829,97 @@
       <c r="A5" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B5" t="s" s="0">
+      <c r="B5" t="s">
         <v>16</v>
       </c>
-      <c r="C5" t="s" s="0">
+      <c r="C5" t="s">
         <v>182</v>
       </c>
-      <c r="D5" t="s" s="0">
+      <c r="D5" t="s">
         <v>183</v>
       </c>
-      <c r="E5" t="s" s="0">
+      <c r="E5" t="s">
         <v>398</v>
       </c>
-      <c r="G5" t="s" s="0">
+      <c r="G5" t="s">
         <v>40</v>
       </c>
-      <c r="H5" t="s" s="0">
+      <c r="H5" t="s">
         <v>17</v>
       </c>
-      <c r="I5" t="s" s="0">
+      <c r="I5" t="s">
         <v>12</v>
       </c>
-      <c r="J5" t="s" s="0">
+      <c r="J5" t="s">
         <v>399</v>
       </c>
-      <c r="K5" t="s" s="0">
+      <c r="K5" t="s">
         <v>126</v>
       </c>
-      <c r="L5" t="s" s="0">
+      <c r="L5" t="s">
         <v>191</v>
       </c>
-      <c r="M5" t="s" s="0">
+      <c r="M5" t="s">
         <v>192</v>
       </c>
-      <c r="N5" t="s" s="0">
+      <c r="N5" t="s">
         <v>128</v>
       </c>
-      <c r="O5" t="s" s="0">
+      <c r="O5" t="s">
         <v>129</v>
       </c>
-      <c r="P5" t="s" s="0">
+      <c r="P5" t="s">
         <v>191</v>
       </c>
-      <c r="Q5" t="s" s="0">
+      <c r="Q5" t="s">
         <v>400</v>
       </c>
-      <c r="R5" t="s" s="0">
+      <c r="R5" t="s">
         <v>211</v>
       </c>
-      <c r="S5" t="s" s="0">
+      <c r="S5" t="s">
         <v>401</v>
       </c>
-      <c r="T5" t="s" s="0">
+      <c r="T5" t="s">
         <v>402</v>
       </c>
-      <c r="U5" t="s" s="0">
+      <c r="U5" t="s">
         <v>403</v>
       </c>
-      <c r="V5" t="s" s="0">
+      <c r="V5" t="s">
         <v>492</v>
       </c>
-      <c r="W5" t="s" s="0">
+      <c r="W5" t="s">
         <v>491</v>
       </c>
-      <c r="X5" t="s" s="0">
+      <c r="X5" t="s">
         <v>404</v>
       </c>
-      <c r="Y5" t="s" s="0">
+      <c r="Y5" t="s">
         <v>12</v>
       </c>
-      <c r="Z5" t="s" s="0">
+      <c r="Z5" t="s">
         <v>405</v>
       </c>
-      <c r="AA5" t="s" s="0">
+      <c r="AA5" t="s">
         <v>249</v>
       </c>
-      <c r="AB5" t="s" s="0">
+      <c r="AB5" t="s">
         <v>406</v>
       </c>
-      <c r="AC5" t="s" s="0">
+      <c r="AC5" t="s">
         <v>19</v>
       </c>
-      <c r="AD5" t="s" s="0">
+      <c r="AD5" t="s">
         <v>37</v>
       </c>
-      <c r="AE5" t="s" s="0">
+      <c r="AE5" t="s">
         <v>407</v>
       </c>
-      <c r="AF5" t="s" s="0">
+      <c r="AF5" t="s">
         <v>408</v>
       </c>
-      <c r="AG5" t="s" s="0">
+      <c r="AG5" t="s">
         <v>12</v>
       </c>
     </row>
@@ -4955,76 +4927,76 @@
       <c r="A6" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="B6" t="s" s="0">
+      <c r="B6" t="s">
         <v>18</v>
       </c>
-      <c r="C6" t="s" s="0">
+      <c r="C6" t="s">
         <v>291</v>
       </c>
-      <c r="D6" t="s" s="0">
+      <c r="D6" t="s">
         <v>292</v>
       </c>
-      <c r="E6" t="s" s="0">
+      <c r="E6" t="s">
         <v>409</v>
       </c>
-      <c r="G6" t="s" s="0">
+      <c r="G6" t="s">
         <v>42</v>
       </c>
-      <c r="H6" t="s" s="0">
+      <c r="H6" t="s">
         <v>19</v>
       </c>
-      <c r="I6" t="s" s="0">
+      <c r="I6" t="s">
         <v>12</v>
       </c>
-      <c r="J6" t="s" s="0">
+      <c r="J6" t="s">
         <v>410</v>
       </c>
-      <c r="K6" t="s" s="0">
+      <c r="K6" t="s">
         <v>411</v>
       </c>
-      <c r="L6" t="s" s="0">
+      <c r="L6" t="s">
         <v>169</v>
       </c>
-      <c r="M6" t="s" s="0">
+      <c r="M6" t="s">
         <v>412</v>
       </c>
-      <c r="N6" t="s" s="0">
+      <c r="N6" t="s">
         <v>128</v>
       </c>
-      <c r="O6" t="s" s="0">
+      <c r="O6" t="s">
         <v>129</v>
       </c>
-      <c r="P6" t="s" s="0">
+      <c r="P6" t="s">
         <v>169</v>
       </c>
-      <c r="Q6" t="s" s="0">
+      <c r="Q6" t="s">
         <v>413</v>
       </c>
-      <c r="R6" t="s" s="0">
+      <c r="R6" t="s">
         <v>251</v>
       </c>
-      <c r="S6" t="s" s="0">
+      <c r="S6" t="s">
         <v>414</v>
       </c>
-      <c r="T6" t="s" s="0">
+      <c r="T6" t="s">
         <v>415</v>
       </c>
-      <c r="U6" t="s" s="0">
+      <c r="U6" t="s">
         <v>416</v>
       </c>
-      <c r="V6" t="s" s="0">
+      <c r="V6" t="s">
         <v>492</v>
       </c>
-      <c r="W6" t="s" s="0">
+      <c r="W6" t="s">
         <v>491</v>
       </c>
-      <c r="X6" t="s" s="0">
+      <c r="X6" t="s">
         <v>417</v>
       </c>
-      <c r="Y6" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="AG6" t="s" s="0">
+      <c r="Y6" t="s">
+        <v>9</v>
+      </c>
+      <c r="AG6" t="s">
         <v>9</v>
       </c>
     </row>
@@ -5032,76 +5004,76 @@
       <c r="A7" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B7" t="s" s="0">
+      <c r="B7" t="s">
         <v>273</v>
       </c>
-      <c r="C7" t="s" s="0">
+      <c r="C7" t="s">
         <v>321</v>
       </c>
-      <c r="D7" t="s" s="0">
+      <c r="D7" t="s">
         <v>322</v>
       </c>
-      <c r="E7" t="s" s="0">
+      <c r="E7" t="s">
         <v>418</v>
       </c>
-      <c r="G7" t="s" s="0">
+      <c r="G7" t="s">
         <v>36</v>
       </c>
-      <c r="H7" t="s" s="0">
+      <c r="H7" t="s">
         <v>8</v>
       </c>
-      <c r="I7" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="J7" t="s" s="0">
+      <c r="I7" t="s">
+        <v>9</v>
+      </c>
+      <c r="J7" t="s">
         <v>419</v>
       </c>
-      <c r="K7" t="s" s="0">
+      <c r="K7" t="s">
         <v>420</v>
       </c>
-      <c r="L7" t="s" s="0">
+      <c r="L7" t="s">
         <v>219</v>
       </c>
-      <c r="M7" t="s" s="0">
+      <c r="M7" t="s">
         <v>220</v>
       </c>
-      <c r="N7" t="s" s="0">
+      <c r="N7" t="s">
         <v>128</v>
       </c>
-      <c r="O7" t="s" s="0">
+      <c r="O7" t="s">
         <v>129</v>
       </c>
-      <c r="P7" t="s" s="0">
+      <c r="P7" t="s">
         <v>498</v>
       </c>
-      <c r="Q7" t="s" s="0">
+      <c r="Q7" t="s">
         <v>421</v>
       </c>
-      <c r="R7" t="s" s="0">
+      <c r="R7" t="s">
         <v>276</v>
       </c>
-      <c r="S7" t="s" s="0">
+      <c r="S7" t="s">
         <v>422</v>
       </c>
-      <c r="T7" t="s" s="0">
+      <c r="T7" t="s">
         <v>423</v>
       </c>
-      <c r="U7" t="s" s="0">
+      <c r="U7" t="s">
         <v>424</v>
       </c>
-      <c r="V7" t="s" s="0">
+      <c r="V7" t="s">
         <v>492</v>
       </c>
-      <c r="W7" t="s" s="0">
+      <c r="W7" t="s">
         <v>491</v>
       </c>
-      <c r="X7" t="s" s="0">
+      <c r="X7" t="s">
         <v>425</v>
       </c>
-      <c r="Y7" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="AG7" t="s" s="0">
+      <c r="Y7" t="s">
+        <v>9</v>
+      </c>
+      <c r="AG7" t="s">
         <v>12</v>
       </c>
     </row>
@@ -5109,76 +5081,76 @@
       <c r="A8" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="B8" t="s" s="0">
+      <c r="B8" t="s">
         <v>290</v>
       </c>
-      <c r="C8" t="s" s="0">
+      <c r="C8" t="s">
         <v>426</v>
       </c>
-      <c r="D8" t="s" s="0">
+      <c r="D8" t="s">
         <v>427</v>
       </c>
-      <c r="E8" t="s" s="0">
+      <c r="E8" t="s">
         <v>428</v>
       </c>
-      <c r="G8" t="s" s="0">
+      <c r="G8" t="s">
         <v>37</v>
       </c>
-      <c r="H8" t="s" s="0">
+      <c r="H8" t="s">
         <v>11</v>
       </c>
-      <c r="I8" t="s" s="0">
+      <c r="I8" t="s">
         <v>12</v>
       </c>
-      <c r="J8" t="s" s="0">
+      <c r="J8" t="s">
         <v>429</v>
       </c>
-      <c r="K8" t="s" s="0">
+      <c r="K8" t="s">
         <v>430</v>
       </c>
-      <c r="L8" t="s" s="0">
+      <c r="L8" t="s">
         <v>284</v>
       </c>
-      <c r="M8" t="s" s="0">
+      <c r="M8" t="s">
         <v>285</v>
       </c>
-      <c r="N8" t="s" s="0">
+      <c r="N8" t="s">
         <v>128</v>
       </c>
-      <c r="O8" t="s" s="0">
+      <c r="O8" t="s">
         <v>129</v>
       </c>
-      <c r="P8" t="s" s="0">
+      <c r="P8" t="s">
         <v>284</v>
       </c>
-      <c r="Q8" t="s" s="0">
+      <c r="Q8" t="s">
         <v>431</v>
       </c>
-      <c r="R8" t="s" s="0">
+      <c r="R8" t="s">
         <v>293</v>
       </c>
-      <c r="S8" t="s" s="0">
+      <c r="S8" t="s">
         <v>432</v>
       </c>
-      <c r="T8" t="s" s="0">
+      <c r="T8" t="s">
         <v>433</v>
       </c>
-      <c r="U8" t="s" s="0">
+      <c r="U8" t="s">
         <v>434</v>
       </c>
-      <c r="V8" t="s" s="0">
+      <c r="V8" t="s">
         <v>492</v>
       </c>
-      <c r="W8" t="s" s="0">
+      <c r="W8" t="s">
         <v>491</v>
       </c>
-      <c r="X8" t="s" s="0">
+      <c r="X8" t="s">
         <v>435</v>
       </c>
-      <c r="Y8" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="AG8" t="s" s="0">
+      <c r="Y8" t="s">
+        <v>9</v>
+      </c>
+      <c r="AG8" t="s">
         <v>9</v>
       </c>
     </row>
@@ -5186,97 +5158,97 @@
       <c r="A9" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="B9" t="s" s="0">
+      <c r="B9" t="s">
         <v>320</v>
       </c>
-      <c r="C9" t="s" s="0">
+      <c r="C9" t="s">
         <v>436</v>
       </c>
-      <c r="D9" t="s" s="0">
+      <c r="D9" t="s">
         <v>437</v>
       </c>
-      <c r="E9" t="s" s="0">
+      <c r="E9" t="s">
         <v>438</v>
       </c>
-      <c r="G9" t="s" s="0">
+      <c r="G9" t="s">
         <v>39</v>
       </c>
-      <c r="H9" t="s" s="0">
+      <c r="H9" t="s">
         <v>15</v>
       </c>
-      <c r="I9" t="s" s="0">
+      <c r="I9" t="s">
         <v>12</v>
       </c>
-      <c r="J9" t="s" s="0">
+      <c r="J9" t="s">
         <v>439</v>
       </c>
-      <c r="K9" t="s" s="0">
+      <c r="K9" t="s">
         <v>440</v>
       </c>
-      <c r="L9" t="s" s="0">
+      <c r="L9" t="s">
         <v>300</v>
       </c>
-      <c r="M9" t="s" s="0">
+      <c r="M9" t="s">
         <v>441</v>
       </c>
-      <c r="N9" t="s" s="0">
+      <c r="N9" t="s">
         <v>128</v>
       </c>
-      <c r="O9" t="s" s="0">
+      <c r="O9" t="s">
         <v>129</v>
       </c>
-      <c r="P9" t="s" s="0">
+      <c r="P9" t="s">
         <v>300</v>
       </c>
-      <c r="Q9" t="s" s="0">
+      <c r="Q9" t="s">
         <v>442</v>
       </c>
-      <c r="R9" t="s" s="0">
+      <c r="R9" t="s">
         <v>323</v>
       </c>
-      <c r="S9" t="s" s="0">
+      <c r="S9" t="s">
         <v>443</v>
       </c>
-      <c r="T9" t="s" s="0">
+      <c r="T9" t="s">
         <v>444</v>
       </c>
-      <c r="U9" t="s" s="0">
+      <c r="U9" t="s">
         <v>445</v>
       </c>
-      <c r="V9" t="s" s="0">
+      <c r="V9" t="s">
         <v>492</v>
       </c>
-      <c r="W9" t="s" s="0">
+      <c r="W9" t="s">
         <v>490</v>
       </c>
-      <c r="X9" t="s" s="0">
+      <c r="X9" t="s">
         <v>446</v>
       </c>
-      <c r="Y9" t="s" s="0">
+      <c r="Y9" t="s">
         <v>12</v>
       </c>
-      <c r="Z9" t="s" s="0">
+      <c r="Z9" t="s">
         <v>447</v>
       </c>
-      <c r="AA9" t="s" s="0">
+      <c r="AA9" t="s">
         <v>119</v>
       </c>
-      <c r="AB9" t="s" s="0">
+      <c r="AB9" t="s">
         <v>448</v>
       </c>
-      <c r="AC9" t="s" s="0">
+      <c r="AC9" t="s">
         <v>449</v>
       </c>
-      <c r="AD9" t="s" s="0">
+      <c r="AD9" t="s">
         <v>39</v>
       </c>
-      <c r="AE9" t="s" s="0">
+      <c r="AE9" t="s">
         <v>450</v>
       </c>
-      <c r="AF9" t="s" s="0">
+      <c r="AF9" t="s">
         <v>451</v>
       </c>
-      <c r="AG9" t="s" s="0">
+      <c r="AG9" t="s">
         <v>9</v>
       </c>
     </row>
@@ -5287,97 +5259,133 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:U2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="5.90625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="6.90625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="11.81640625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="10.81640625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="23.6328125"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="9.7265625"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="11.36328125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="12.6328125"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="3.81640625"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="8.36328125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="7.7265625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="7.90625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="10.54296875"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="7.36328125"/>
+    <col min="1" max="1" width="5.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.6328125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.6328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="3.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.36328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="7.90625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="7.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" t="s" s="0">
+    <row r="1" spans="1:21" ht="17" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>363</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>57</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>452</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s">
         <v>453</v>
       </c>
-      <c r="G1" t="s" s="0">
+      <c r="G1" t="s">
         <v>454</v>
       </c>
-      <c r="H1" t="s" s="0">
+      <c r="H1" t="s">
         <v>26</v>
       </c>
-      <c r="I1" t="s" s="0">
+      <c r="I1" t="s">
         <v>455</v>
       </c>
-      <c r="J1" t="s" s="0">
+      <c r="J1" t="s">
         <v>456</v>
       </c>
-      <c r="K1" t="s" s="0">
+      <c r="K1" t="s">
         <v>457</v>
       </c>
-      <c r="L1" t="s" s="0">
+      <c r="L1" t="s">
         <v>458</v>
       </c>
-      <c r="M1" t="s" s="0">
+      <c r="M1" t="s">
         <v>459</v>
       </c>
-      <c r="N1" t="s" s="0">
+      <c r="N1" t="s">
         <v>460</v>
       </c>
-      <c r="O1" t="s" s="0">
+      <c r="O1" t="s">
         <v>504</v>
       </c>
+      <c r="P1" t="s">
+        <v>516</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>517</v>
+      </c>
+      <c r="R1" t="s">
+        <v>518</v>
+      </c>
+      <c r="S1" t="s">
+        <v>100</v>
+      </c>
+      <c r="T1" t="s">
+        <v>521</v>
+      </c>
+      <c r="U1" t="s">
+        <v>522</v>
+      </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.35">
-      <c r="A2" s="29" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" t="s" s="0">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.35">
+      <c r="A2" s="31" t="s">
+        <v>513</v>
+      </c>
+      <c r="B2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" t="s" s="0">
+      <c r="C2" t="s">
         <v>490</v>
       </c>
-      <c r="D2" s="0">
-        <v>6369029084</v>
-      </c>
-      <c r="E2" t="s" s="0">
+      <c r="D2">
+        <v>9965331986</v>
+      </c>
+      <c r="E2" t="s">
+        <v>528</v>
+      </c>
+      <c r="H2" t="s">
+        <v>249</v>
+      </c>
+      <c r="I2" t="s">
+        <v>9</v>
+      </c>
+      <c r="N2" t="s">
+        <v>461</v>
+      </c>
+      <c r="P2" t="s">
+        <v>526</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>519</v>
+      </c>
+      <c r="R2" t="s">
+        <v>520</v>
+      </c>
+      <c r="S2" s="29" t="s">
         <v>523</v>
       </c>
-      <c r="H2" t="s" s="0">
-        <v>249</v>
-      </c>
-      <c r="I2" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="N2" t="s" s="0">
-        <v>461</v>
+      <c r="T2" t="s">
+        <v>519</v>
+      </c>
+      <c r="U2" t="s">
+        <v>519</v>
       </c>
     </row>
   </sheetData>
@@ -5392,275 +5400,275 @@
   <dimension ref="A1:AN5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="5.90625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="6.90625"/>
-    <col min="3" max="3" bestFit="true" customWidth="true" width="14.54296875"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="15.26953125"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="11.81640625"/>
-    <col min="6" max="6" bestFit="true" customWidth="true" width="9.0"/>
-    <col min="7" max="7" bestFit="true" customWidth="true" width="7.54296875"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="4.81640625"/>
-    <col min="9" max="9" bestFit="true" customWidth="true" width="10.08984375"/>
-    <col min="10" max="10" bestFit="true" customWidth="true" width="9.36328125"/>
-    <col min="11" max="11" bestFit="true" customWidth="true" width="4.81640625"/>
-    <col min="12" max="12" bestFit="true" customWidth="true" width="6.7265625"/>
-    <col min="13" max="13" bestFit="true" customWidth="true" width="6.81640625"/>
-    <col min="14" max="14" bestFit="true" customWidth="true" width="11.1796875"/>
-    <col min="15" max="15" bestFit="true" customWidth="true" width="10.54296875"/>
-    <col min="16" max="16" bestFit="true" customWidth="true" width="10.08984375"/>
-    <col min="17" max="17" bestFit="true" customWidth="true" width="7.90625"/>
-    <col min="18" max="18" bestFit="true" customWidth="true" width="10.36328125"/>
-    <col min="19" max="19" bestFit="true" customWidth="true" width="12.08984375"/>
-    <col min="20" max="20" bestFit="true" customWidth="true" width="5.81640625"/>
-    <col min="21" max="21" bestFit="true" customWidth="true" width="10.6328125"/>
-    <col min="22" max="22" bestFit="true" customWidth="true" width="12.54296875"/>
-    <col min="23" max="23" bestFit="true" customWidth="true" width="10.81640625"/>
-    <col min="24" max="24" bestFit="true" customWidth="true" width="8.54296875"/>
-    <col min="25" max="25" bestFit="true" customWidth="true" width="9.81640625"/>
-    <col min="26" max="26" bestFit="true" customWidth="true" width="8.81640625"/>
-    <col min="27" max="27" bestFit="true" customWidth="true" width="10.36328125"/>
-    <col min="28" max="28" bestFit="true" customWidth="true" width="7.54296875"/>
-    <col min="29" max="29" bestFit="true" customWidth="true" width="11.81640625"/>
-    <col min="30" max="30" bestFit="true" customWidth="true" width="12.1796875"/>
-    <col min="31" max="31" customWidth="true" width="12.1796875"/>
-    <col min="32" max="32" bestFit="true" customWidth="true" width="19.81640625"/>
-    <col min="35" max="35" bestFit="true" customWidth="true" width="11.6328125"/>
-    <col min="38" max="38" bestFit="true" customWidth="true" width="12.90625"/>
+    <col min="1" max="1" width="5.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6.90625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.54296875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.54296875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="4.81640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.36328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="4.81640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="6.7265625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="6.81640625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.08984375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="7.90625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="12.08984375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="5.81640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="10.6328125" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="10.81640625" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="8.54296875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="9.81640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="7.54296875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="12.1796875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="12.1796875" customWidth="1"/>
+    <col min="32" max="32" width="19.81640625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="12.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:40" x14ac:dyDescent="0.35">
-      <c r="A1" t="s" s="0">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s" s="0">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s" s="0">
+      <c r="C1" t="s">
         <v>462</v>
       </c>
-      <c r="D1" t="s" s="0">
+      <c r="D1" t="s">
         <v>463</v>
       </c>
-      <c r="E1" t="s" s="0">
+      <c r="E1" t="s">
         <v>363</v>
       </c>
-      <c r="F1" t="s" s="0">
+      <c r="F1" t="s">
         <v>26</v>
       </c>
-      <c r="G1" t="s" s="0">
+      <c r="G1" t="s">
         <v>464</v>
       </c>
-      <c r="H1" t="s" s="0">
+      <c r="H1" t="s">
         <v>465</v>
       </c>
-      <c r="I1" t="s" s="0">
+      <c r="I1" t="s">
         <v>466</v>
       </c>
-      <c r="J1" t="s" s="0">
+      <c r="J1" t="s">
         <v>467</v>
       </c>
-      <c r="K1" t="s" s="0">
+      <c r="K1" t="s">
         <v>468</v>
       </c>
-      <c r="L1" t="s" s="0">
+      <c r="L1" t="s">
         <v>469</v>
       </c>
-      <c r="M1" t="s" s="0">
+      <c r="M1" t="s">
         <v>470</v>
       </c>
-      <c r="N1" t="s" s="0">
+      <c r="N1" t="s">
         <v>471</v>
       </c>
-      <c r="O1" t="s" s="0">
+      <c r="O1" t="s">
         <v>472</v>
       </c>
-      <c r="P1" t="s" s="0">
+      <c r="P1" t="s">
         <v>473</v>
       </c>
-      <c r="Q1" t="s" s="0">
+      <c r="Q1" t="s">
         <v>474</v>
       </c>
-      <c r="R1" t="s" s="0">
+      <c r="R1" t="s">
         <v>475</v>
       </c>
-      <c r="S1" t="s" s="0">
+      <c r="S1" t="s">
         <v>476</v>
       </c>
-      <c r="T1" t="s" s="0">
+      <c r="T1" t="s">
         <v>477</v>
       </c>
-      <c r="U1" t="s" s="0">
+      <c r="U1" t="s">
         <v>478</v>
       </c>
-      <c r="V1" t="s" s="0">
+      <c r="V1" t="s">
         <v>479</v>
       </c>
-      <c r="W1" t="s" s="0">
+      <c r="W1" t="s">
         <v>480</v>
       </c>
-      <c r="X1" t="s" s="0">
+      <c r="X1" t="s">
         <v>481</v>
       </c>
-      <c r="Y1" t="s" s="0">
+      <c r="Y1" t="s">
         <v>482</v>
       </c>
-      <c r="Z1" t="s" s="0">
+      <c r="Z1" t="s">
         <v>483</v>
       </c>
-      <c r="AA1" t="s" s="0">
+      <c r="AA1" t="s">
         <v>484</v>
       </c>
-      <c r="AB1" t="s" s="0">
+      <c r="AB1" t="s">
         <v>500</v>
       </c>
-      <c r="AC1" t="s" s="0">
+      <c r="AC1" t="s">
         <v>501</v>
       </c>
-      <c r="AD1" t="s" s="0">
+      <c r="AD1" t="s">
         <v>502</v>
       </c>
-      <c r="AE1" t="s" s="0">
+      <c r="AE1" t="s">
         <v>505</v>
       </c>
-      <c r="AF1" t="s" s="0">
+      <c r="AF1" t="s">
         <v>503</v>
       </c>
-      <c r="AG1" t="s" s="0">
+      <c r="AG1" t="s">
         <v>507</v>
       </c>
-      <c r="AH1" t="s" s="0">
+      <c r="AH1" t="s">
         <v>515</v>
       </c>
-      <c r="AI1" t="s" s="0">
+      <c r="AI1" t="s">
         <v>516</v>
       </c>
-      <c r="AJ1" t="s" s="0">
-        <v>519</v>
-      </c>
-      <c r="AK1" t="s" s="0">
-        <v>520</v>
-      </c>
-      <c r="AL1" t="s" s="0">
+      <c r="AJ1" t="s">
+        <v>517</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>518</v>
+      </c>
+      <c r="AL1" t="s">
         <v>100</v>
       </c>
-      <c r="AM1" t="s" s="0">
-        <v>524</v>
-      </c>
-      <c r="AN1" t="s" s="0">
-        <v>525</v>
+      <c r="AM1" t="s">
+        <v>521</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>522</v>
       </c>
     </row>
     <row r="2" spans="1:40" x14ac:dyDescent="0.35">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="30" t="s">
         <v>513</v>
       </c>
-      <c r="B2" t="s" s="0">
+      <c r="B2" t="s">
         <v>485</v>
       </c>
-      <c r="C2" s="0">
+      <c r="C2">
         <v>9965331986</v>
       </c>
-      <c r="D2" t="s" s="0">
-        <v>531</v>
-      </c>
-      <c r="E2" t="s" s="0">
+      <c r="D2" t="s">
+        <v>527</v>
+      </c>
+      <c r="E2" t="s">
         <v>490</v>
       </c>
-      <c r="F2" t="s" s="0">
+      <c r="F2" t="s">
         <v>370</v>
       </c>
-      <c r="G2" s="0">
+      <c r="G2">
         <v>1000</v>
       </c>
-      <c r="H2" s="0">
+      <c r="H2">
         <v>100</v>
       </c>
-      <c r="I2" t="s" s="0">
+      <c r="I2" t="s">
         <v>12</v>
       </c>
-      <c r="J2" t="s" s="0">
+      <c r="J2" t="s">
         <v>486</v>
       </c>
-      <c r="K2" t="s" s="0">
+      <c r="K2" t="s">
         <v>487</v>
       </c>
-      <c r="M2" s="0">
+      <c r="M2">
         <v>20309</v>
       </c>
-      <c r="N2" s="0">
+      <c r="N2">
         <v>600</v>
       </c>
-      <c r="O2" s="0">
+      <c r="O2">
         <v>73830</v>
       </c>
-      <c r="P2" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="Q2" t="s" s="0">
+      <c r="P2" t="s">
+        <v>9</v>
+      </c>
+      <c r="Q2" t="s">
         <v>488</v>
       </c>
-      <c r="R2" t="s" s="0">
+      <c r="R2" t="s">
         <v>489</v>
       </c>
       <c r="S2" s="2">
         <v>46146</v>
       </c>
-      <c r="T2" s="0">
+      <c r="T2">
         <v>39480</v>
       </c>
-      <c r="V2" t="s" s="0">
+      <c r="V2" t="s">
         <v>12</v>
       </c>
       <c r="W2" s="2">
         <v>46167</v>
       </c>
-      <c r="X2" t="s" s="0">
-        <v>528</v>
-      </c>
-      <c r="Y2" s="0">
+      <c r="X2" t="s">
+        <v>525</v>
+      </c>
+      <c r="Y2">
         <v>93209</v>
       </c>
-      <c r="Z2" s="0">
+      <c r="Z2">
         <v>2093002</v>
       </c>
-      <c r="AA2" s="0">
+      <c r="AA2">
         <v>300</v>
       </c>
-      <c r="AB2" t="s" s="0">
-        <v>9</v>
-      </c>
-      <c r="AC2" s="0">
+      <c r="AB2" t="s">
+        <v>9</v>
+      </c>
+      <c r="AC2">
         <v>124356</v>
       </c>
-      <c r="AD2" s="0">
+      <c r="AD2">
         <v>0</v>
       </c>
-      <c r="AE2" s="0">
+      <c r="AE2">
         <v>0</v>
       </c>
-      <c r="AF2" t="s" s="0">
+      <c r="AF2" t="s">
         <v>506</v>
       </c>
-      <c r="AG2" s="0">
+      <c r="AG2">
         <v>1000</v>
       </c>
-      <c r="AI2" t="s" s="0">
-        <v>529</v>
-      </c>
-      <c r="AJ2" t="s" s="0">
-        <v>521</v>
-      </c>
-      <c r="AK2" t="s" s="0">
-        <v>522</v>
-      </c>
-      <c r="AL2" s="30" t="s">
+      <c r="AI2" t="s">
         <v>526</v>
       </c>
-      <c r="AM2" t="s" s="0">
-        <v>521</v>
-      </c>
-      <c r="AN2" t="s" s="0">
-        <v>521</v>
+      <c r="AJ2" t="s">
+        <v>519</v>
+      </c>
+      <c r="AK2" t="s">
+        <v>520</v>
+      </c>
+      <c r="AL2" s="29" t="s">
+        <v>523</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>519</v>
+      </c>
+      <c r="AN2" t="s">
+        <v>519</v>
       </c>
     </row>
     <row r="5" spans="1:40" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Scroll has been done in customer creation
</commit_message>
<xml_diff>
--- a/kalarakal_updated.xlsx
+++ b/kalarakal_updated.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="797" uniqueCount="423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="808" uniqueCount="424">
   <si>
     <t>Status</t>
   </si>
@@ -1298,6 +1298,9 @@
   </si>
   <si>
     <t>12 Sec</t>
+  </si>
+  <si>
+    <t>10 Sec</t>
   </si>
 </sst>
 </file>
@@ -1305,7 +1308,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="36" x14ac:knownFonts="1">
+  <fonts count="45" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1525,6 +1528,60 @@
       <b val="true"/>
       <color indexed="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11.0"/>
+      <b val="true"/>
+      <color indexed="17"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1547,7 +1604,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
@@ -1589,6 +1646,15 @@
     <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="0" applyFont="true"/>
+    <xf numFmtId="0" fontId="44" fillId="0" borderId="0" xfId="0" applyFont="true"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1901,7 +1967,7 @@
         <v>388</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>422</v>
+        <v>423</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -2067,7 +2133,7 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="39" t="s">
         <v>391</v>
       </c>
       <c r="B2" t="s" s="0">
@@ -2653,7 +2719,7 @@
       </c>
     </row>
     <row r="2" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="35" t="s">
+      <c r="A2" s="40" t="s">
         <v>6</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -2767,7 +2833,7 @@
       </c>
     </row>
     <row r="3" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="36" t="s">
+      <c r="A3" s="41" t="s">
         <v>6</v>
       </c>
       <c r="B3" s="3" t="s">
@@ -2859,7 +2925,7 @@
       <c r="AN3" s="3"/>
     </row>
     <row r="4" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="37" t="s">
+      <c r="A4" s="42" t="s">
         <v>6</v>
       </c>
       <c r="B4" s="3" t="s">
@@ -2967,7 +3033,7 @@
       <c r="AN4" s="3"/>
     </row>
     <row r="5" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="38" t="s">
+      <c r="A5" s="43" t="s">
         <v>391</v>
       </c>
       <c r="B5" s="3" t="s">
@@ -3091,7 +3157,9 @@
       </c>
     </row>
     <row r="6" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="3"/>
+      <c r="A6" s="44" t="s">
+        <v>6</v>
+      </c>
       <c r="B6" s="3" t="s">
         <v>18</v>
       </c>
@@ -3185,7 +3253,9 @@
       <c r="AN6" s="3"/>
     </row>
     <row r="7" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="3"/>
+      <c r="A7" s="45" t="s">
+        <v>6</v>
+      </c>
       <c r="B7" s="3" t="s">
         <v>179</v>
       </c>
@@ -3275,7 +3345,9 @@
       <c r="AN7" s="3"/>
     </row>
     <row r="8" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="3"/>
+      <c r="A8" s="46" t="s">
+        <v>391</v>
+      </c>
       <c r="B8" s="3" t="s">
         <v>193</v>
       </c>
@@ -3385,7 +3457,9 @@
       </c>
     </row>
     <row r="9" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="3"/>
+      <c r="A9" s="47" t="s">
+        <v>6</v>
+      </c>
       <c r="B9" s="3" t="s">
         <v>210</v>
       </c>

</xml_diff>

<commit_message>
profession close button changed
</commit_message>
<xml_diff>
--- a/kalarakal_updated.xlsx
+++ b/kalarakal_updated.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chella\eclipse-workspace\mavenCrm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BD02960-0AD0-4C52-9A61-5EB415E38DD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5275A366-2466-43E4-A045-853496D17BA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="806" uniqueCount="427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="801" uniqueCount="430">
   <si>
     <t>Status</t>
   </si>
@@ -1156,9 +1156,6 @@
     <t>Asst manager</t>
   </si>
   <si>
-    <t>23 Sec</t>
-  </si>
-  <si>
     <t>Tirupur</t>
   </si>
   <si>
@@ -1198,18 +1195,9 @@
     <t>0 Pass 1 Fail</t>
   </si>
   <si>
-    <t>21 Sec</t>
-  </si>
-  <si>
-    <t>87 Sec</t>
-  </si>
-  <si>
     <t>FAIL</t>
   </si>
   <si>
-    <t>18 Sec</t>
-  </si>
-  <si>
     <t>accNo</t>
   </si>
   <si>
@@ -1237,9 +1225,6 @@
     <t>738920390989</t>
   </si>
   <si>
-    <t>27 Sec</t>
-  </si>
-  <si>
     <t>HDFC</t>
   </si>
   <si>
@@ -1249,67 +1234,91 @@
     <t>DG-not allocated</t>
   </si>
   <si>
-    <t>Digi silver</t>
+    <t>Ukkadam</t>
+  </si>
+  <si>
+    <t>Madurai west</t>
+  </si>
+  <si>
+    <t>Sowcarpet</t>
+  </si>
+  <si>
+    <t>Erode East</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Salem Bazaar </t>
+  </si>
+  <si>
+    <t>Dindigul Fort</t>
+  </si>
+  <si>
+    <t>Raj@1233</t>
+  </si>
+  <si>
+    <t>PanNo</t>
+  </si>
+  <si>
+    <t>VoterId</t>
+  </si>
+  <si>
+    <t>rationCard</t>
+  </si>
+  <si>
+    <t>nominieeImage</t>
+  </si>
+  <si>
+    <t>AAAPL1234C</t>
+  </si>
+  <si>
+    <t>1234 5678 9012</t>
+  </si>
+  <si>
+    <t>TN123456789012</t>
+  </si>
+  <si>
+    <t>tirupur</t>
+  </si>
+  <si>
+    <t>2 Pass 0 Fail</t>
+  </si>
+  <si>
+    <t>207 Sec</t>
+  </si>
+  <si>
+    <t>25 Sec</t>
+  </si>
+  <si>
+    <t>26 Sec</t>
+  </si>
+  <si>
+    <t>22 Sec</t>
+  </si>
+  <si>
+    <t>200 Sec</t>
+  </si>
+  <si>
+    <t>14 Sec</t>
+  </si>
+  <si>
+    <t>1 Pass 0 Fail</t>
+  </si>
+  <si>
+    <t>34 Sec</t>
+  </si>
+  <si>
+    <t>19 Sec</t>
+  </si>
+  <si>
+    <t>12 Sec</t>
   </si>
   <si>
     <t>36 Sec</t>
   </si>
   <si>
-    <t>Ukkadam</t>
-  </si>
-  <si>
-    <t>Madurai west</t>
-  </si>
-  <si>
-    <t>Sowcarpet</t>
-  </si>
-  <si>
-    <t>Erode East</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Salem Bazaar </t>
-  </si>
-  <si>
-    <t>Dindigul Fort</t>
-  </si>
-  <si>
-    <t>Raj@1233</t>
-  </si>
-  <si>
-    <t>PanNo</t>
-  </si>
-  <si>
-    <t>VoterId</t>
-  </si>
-  <si>
-    <t>rationCard</t>
-  </si>
-  <si>
-    <t>nominieeImage</t>
-  </si>
-  <si>
-    <t>AAAPL1234C</t>
-  </si>
-  <si>
-    <t>1234 5678 9012</t>
-  </si>
-  <si>
-    <t>TN123456789012</t>
-  </si>
-  <si>
-    <t>10 Sec</t>
-  </si>
-  <si>
-    <t>tirupur</t>
-  </si>
-  <si>
-    <t>2 Pass 0 Fail</t>
-  </si>
-  <si>
-    <t>207 Sec</t>
-  </si>
-  <si>
-    <t>11 Sec</t>
+    <t>26-DG-38</t>
+  </si>
+  <si>
+    <t>66 Sec</t>
   </si>
 </sst>
 </file>
@@ -1480,19 +1489,19 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color indexed="10"/>
+      <color indexed="17"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <color indexed="10"/>
+      <color indexed="17"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
-      <color indexed="10"/>
+      <color indexed="17"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -1546,7 +1555,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color indexed="17"/>
+      <color indexed="10"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -1559,13 +1568,13 @@
       <name val="Calibri"/>
       <sz val="11.0"/>
       <b val="true"/>
-      <color indexed="10"/>
+      <color indexed="17"/>
     </font>
     <font>
       <name val="Calibri"/>
       <sz val="11.0"/>
       <b val="true"/>
-      <color indexed="10"/>
+      <color indexed="17"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1598,6 +1607,7 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1621,7 +1631,6 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1945,7 +1954,7 @@
         <v>12</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>388</v>
+        <v>387</v>
       </c>
       <c r="D2" t="s" s="0">
         <v>426</v>
@@ -1956,13 +1965,13 @@
         <v>2</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C3" t="s" s="0">
         <v>373</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>389</v>
+        <v>418</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -1970,13 +1979,13 @@
         <v>34</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C4" t="s" s="0">
         <v>373</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>375</v>
+        <v>419</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
@@ -1984,13 +1993,13 @@
         <v>24</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C5" t="s" s="0">
         <v>373</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>392</v>
+        <v>420</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
@@ -2001,10 +2010,10 @@
         <v>9</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>424</v>
+        <v>416</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>425</v>
+        <v>417</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -2015,10 +2024,10 @@
         <v>9</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>390</v>
+        <v>421</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -2029,10 +2038,10 @@
         <v>12</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>388</v>
+        <v>423</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>407</v>
+        <v>427</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -2043,10 +2052,10 @@
         <v>12</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>388</v>
+        <v>423</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>402</v>
+        <v>429</v>
       </c>
     </row>
   </sheetData>
@@ -2056,10 +2065,10 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF37BC37-2A10-492F-B32A-B95007897491}">
-  <dimension ref="A3:AR15"/>
+  <dimension ref="A3:O3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="3" spans="1:44" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>6</v>
       </c>
@@ -2070,10 +2079,10 @@
         <v>368</v>
       </c>
       <c r="E3" t="s" s="0">
+        <v>385</v>
+      </c>
+      <c r="H3" t="s" s="0">
         <v>386</v>
-      </c>
-      <c r="H3" t="s" s="0">
-        <v>387</v>
       </c>
       <c r="I3" t="s" s="0">
         <v>9</v>
@@ -2085,628 +2094,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="32" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="J8" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="K8" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="L8" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="M8" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="N8" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="O8" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="P8" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="Q8" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="R8" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="S8" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="T8" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="U8" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="V8" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="W8" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="X8" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="Y8" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="Z8" s="3"/>
-      <c r="AA8" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="AB8" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="AC8" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="AD8" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="AE8" s="3" t="s">
-        <v>108</v>
-      </c>
-      <c r="AF8" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="AG8" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="AH8" s="1" t="s">
-        <v>414</v>
-      </c>
-      <c r="AI8" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="AJ8" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="AK8" s="3"/>
-      <c r="AL8" s="3"/>
-      <c r="AM8" s="3"/>
-      <c r="AN8" s="3"/>
-      <c r="AO8" t="s" s="0">
-        <v>419</v>
-      </c>
-      <c r="AR8" t="s" s="0">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="9" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="33" t="s">
-        <v>6</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>110</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="G9" s="3"/>
-      <c r="H9" s="3"/>
-      <c r="I9" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="J9" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="K9" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="L9" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="M9" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="N9" s="3" t="s">
-        <v>115</v>
-      </c>
-      <c r="O9" s="3" t="s">
-        <v>116</v>
-      </c>
-      <c r="P9" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="Q9" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="R9" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="S9" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="T9" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="U9" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="V9" s="3" t="s">
-        <v>408</v>
-      </c>
-      <c r="W9" s="3"/>
-      <c r="X9" s="3"/>
-      <c r="Y9" s="3"/>
-      <c r="Z9" s="3"/>
-      <c r="AA9" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="AB9" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="AC9" s="3"/>
-      <c r="AD9" s="3"/>
-      <c r="AE9" s="3"/>
-      <c r="AF9" s="3"/>
-      <c r="AG9" s="3"/>
-      <c r="AH9" s="3" t="s">
-        <v>120</v>
-      </c>
-      <c r="AI9" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="AJ9" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="AK9" s="3"/>
-      <c r="AL9" s="3"/>
-      <c r="AM9" s="3"/>
-      <c r="AN9" s="3"/>
-    </row>
-    <row r="10" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="34" t="s">
-        <v>6</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="I10" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="J10" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="K10" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="L10" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="M10" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="N10" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="O10" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="P10" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="Q10" s="3"/>
-      <c r="R10" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="S10" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="T10" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="U10" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="V10" s="3" t="s">
-        <v>409</v>
-      </c>
-      <c r="W10" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="X10" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="Y10" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="Z10" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="AA10" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="AB10" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="AC10" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="AD10" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="AE10" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="AF10" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="AG10" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="AH10" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="AI10" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="AJ10" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="AK10" s="3"/>
-      <c r="AL10" s="3"/>
-      <c r="AM10" s="3"/>
-      <c r="AN10" s="3"/>
-    </row>
-    <row r="12" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="35" t="s">
-        <v>6</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="K12" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="L12" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="M12" s="3" t="s">
-        <v>169</v>
-      </c>
-      <c r="N12" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="O12" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="P12" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="Q12" s="3"/>
-      <c r="R12" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="S12" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="T12" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="U12" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="V12" s="3" t="s">
-        <v>410</v>
-      </c>
-      <c r="W12" s="3" t="s">
-        <v>175</v>
-      </c>
-      <c r="X12" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="Y12" s="3" t="s">
-        <v>176</v>
-      </c>
-      <c r="Z12" s="3"/>
-      <c r="AA12" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="AB12" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="AC12" s="3"/>
-      <c r="AD12" s="3"/>
-      <c r="AE12" s="3"/>
-      <c r="AF12" s="3"/>
-      <c r="AG12" s="3"/>
-      <c r="AH12" s="3" t="s">
-        <v>178</v>
-      </c>
-      <c r="AI12" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="AJ12" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="AK12" s="3"/>
-      <c r="AL12" s="3"/>
-      <c r="AM12" s="3"/>
-      <c r="AN12" s="3"/>
-    </row>
-    <row r="13" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="36" t="s">
-        <v>6</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>179</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>109</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>180</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>181</v>
-      </c>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-      <c r="I13" s="3" t="s">
-        <v>182</v>
-      </c>
-      <c r="J13" s="3" t="s">
-        <v>183</v>
-      </c>
-      <c r="K13" s="3" t="s">
-        <v>184</v>
-      </c>
-      <c r="L13" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="M13" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="N13" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="O13" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="P13" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="Q13" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="R13" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="S13" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="T13" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="U13" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="V13" s="3" t="s">
-        <v>411</v>
-      </c>
-      <c r="W13" s="3"/>
-      <c r="X13" s="3"/>
-      <c r="Y13" s="3"/>
-      <c r="Z13" s="3"/>
-      <c r="AA13" s="3" t="s">
-        <v>177</v>
-      </c>
-      <c r="AB13" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="AC13" s="3"/>
-      <c r="AD13" s="3"/>
-      <c r="AE13" s="3"/>
-      <c r="AF13" s="3"/>
-      <c r="AG13" s="3"/>
-      <c r="AH13" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="AI13" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="AJ13" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="AK13" s="3"/>
-      <c r="AL13" s="3"/>
-      <c r="AM13" s="3"/>
-      <c r="AN13" s="3"/>
-    </row>
-    <row r="15" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="37" t="s">
-        <v>6</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>210</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="I15" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="J15" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="K15" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="L15" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="M15" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="N15" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="O15" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="P15" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="Q15" s="3"/>
-      <c r="R15" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="S15" s="3" t="s">
-        <v>100</v>
-      </c>
-      <c r="T15" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="U15" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="V15" s="3" t="s">
-        <v>413</v>
-      </c>
-      <c r="W15" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="X15" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="Y15" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="Z15" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="AA15" s="3" t="s">
-        <v>105</v>
-      </c>
-      <c r="AB15" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="AC15" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="AD15" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="AE15" s="3" t="s">
-        <v>225</v>
-      </c>
-      <c r="AF15" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="AG15" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="AH15" s="3" t="s">
-        <v>226</v>
-      </c>
-      <c r="AI15" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="AJ15" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="AK15" s="3" t="s">
-        <v>227</v>
-      </c>
-      <c r="AL15" s="3" t="s">
-        <v>228</v>
-      </c>
-      <c r="AM15" s="3" t="s">
-        <v>229</v>
-      </c>
-      <c r="AN15" s="3" t="s">
-        <v>230</v>
-      </c>
-    </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="AH8" r:id="rId1" xr:uid="{939D6BFA-866E-47FE-A167-60E9B33C4530}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2741,8 +2129,8 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" s="42" t="s">
-        <v>391</v>
+      <c r="A2" s="41" t="s">
+        <v>388</v>
       </c>
       <c r="B2" t="s" s="0">
         <v>7</v>
@@ -2797,8 +2185,8 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="43" t="s">
-        <v>391</v>
+      <c r="A2" s="15" t="s">
+        <v>6</v>
       </c>
       <c r="B2" t="s" s="0">
         <v>7</v>
@@ -2814,7 +2202,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="14" t="s">
+      <c r="A3" s="16" t="s">
         <v>6</v>
       </c>
       <c r="B3" t="s" s="0">
@@ -2834,7 +2222,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="17" t="s">
         <v>6</v>
       </c>
       <c r="B4" t="s" s="0">
@@ -2851,7 +2239,7 @@
       </c>
     </row>
     <row r="5" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="16" t="s">
+      <c r="A5" s="18" t="s">
         <v>6</v>
       </c>
       <c r="B5" t="s" s="0">
@@ -2871,7 +2259,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="19" t="s">
         <v>6</v>
       </c>
       <c r="B6" t="s" s="0">
@@ -2924,7 +2312,7 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="20" t="s">
         <v>6</v>
       </c>
       <c r="B2" t="s" s="0">
@@ -2941,7 +2329,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="19" t="s">
+      <c r="A3" s="21" t="s">
         <v>6</v>
       </c>
       <c r="B3" t="s" s="0">
@@ -2961,7 +2349,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="22" t="s">
         <v>6</v>
       </c>
       <c r="B4" t="s" s="0">
@@ -2978,7 +2366,7 @@
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="21" t="s">
+      <c r="A5" s="23" t="s">
         <v>6</v>
       </c>
       <c r="B5" t="s" s="0">
@@ -2998,7 +2386,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="24" t="s">
         <v>6</v>
       </c>
       <c r="B6" t="s" s="0">
@@ -3051,7 +2439,7 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="25" t="s">
         <v>6</v>
       </c>
       <c r="B2" t="s" s="0">
@@ -3068,7 +2456,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="24" t="s">
+      <c r="A3" s="26" t="s">
         <v>6</v>
       </c>
       <c r="B3" t="s" s="0">
@@ -3088,7 +2476,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="27" t="s">
         <v>6</v>
       </c>
       <c r="B4" t="s" s="0">
@@ -3105,7 +2493,7 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="26" t="s">
+      <c r="A5" s="28" t="s">
         <v>6</v>
       </c>
       <c r="B5" t="s" s="0">
@@ -3125,7 +2513,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="27" t="s">
+      <c r="A6" s="29" t="s">
         <v>6</v>
       </c>
       <c r="B6" t="s" s="0">
@@ -3145,7 +2533,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:AR3"/>
+  <dimension ref="A1:AR9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" bestFit="true" customWidth="true" width="5.90625"/>
@@ -3314,24 +2702,22 @@
         <v>86</v>
       </c>
       <c r="AO1" t="s" s="0">
-        <v>415</v>
+        <v>408</v>
       </c>
       <c r="AP1" t="s" s="0">
-        <v>416</v>
+        <v>409</v>
       </c>
       <c r="AQ1" t="s" s="0">
-        <v>417</v>
+        <v>410</v>
       </c>
       <c r="AR1" t="s" s="0">
-        <v>418</v>
+        <v>411</v>
       </c>
     </row>
     <row r="2" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="39" t="s">
-        <v>6</v>
-      </c>
+      <c r="A2" s="13"/>
       <c r="B2" s="3" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>87</v>
@@ -3381,13 +2767,13 @@
         <v>100</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="U2" s="3" t="s">
         <v>151</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>423</v>
+        <v>415</v>
       </c>
       <c r="W2" s="3" t="s">
         <v>152</v>
@@ -3444,18 +2830,16 @@
         <v>162</v>
       </c>
       <c r="AP2" t="s" s="0">
-        <v>420</v>
+        <v>413</v>
       </c>
       <c r="AR2" t="s" s="0">
-        <v>397</v>
+        <v>393</v>
       </c>
     </row>
     <row r="3" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="40" t="s">
-        <v>6</v>
-      </c>
+      <c r="A3" s="14"/>
       <c r="B3" s="3" t="s">
-        <v>193</v>
+        <v>10</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>87</v>
@@ -3509,7 +2893,7 @@
         <v>204</v>
       </c>
       <c r="V3" s="3" t="s">
-        <v>412</v>
+        <v>405</v>
       </c>
       <c r="W3" s="3" t="s">
         <v>102</v>
@@ -3556,13 +2940,623 @@
       <c r="AM3" s="3"/>
       <c r="AN3" s="3"/>
       <c r="AQ3" t="s" s="0">
-        <v>421</v>
+        <v>414</v>
       </c>
       <c r="AR3" t="s" s="0">
-        <v>397</v>
+        <v>393</v>
+      </c>
+    </row>
+    <row r="4" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="7"/>
+      <c r="B4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="O4" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="P4" s="3" t="s">
+        <v>97</v>
+      </c>
+      <c r="Q4" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="R4" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="S4" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="T4" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="U4" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="V4" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="W4" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="X4" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="Y4" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="Z4" s="3"/>
+      <c r="AA4" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="AB4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="AC4" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="AD4" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="AE4" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="AF4" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="AG4" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="AH4" s="1" t="s">
+        <v>407</v>
+      </c>
+      <c r="AI4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="AJ4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="AK4" s="3"/>
+      <c r="AL4" s="3"/>
+      <c r="AM4" s="3"/>
+      <c r="AN4" s="3"/>
+      <c r="AO4" t="s" s="0">
+        <v>412</v>
+      </c>
+      <c r="AR4" t="s" s="0">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="5" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="8"/>
+      <c r="B5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3" t="s">
+        <v>112</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="N5" s="3" t="s">
+        <v>115</v>
+      </c>
+      <c r="O5" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="P5" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="Q5" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="R5" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="S5" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="T5" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="U5" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="V5" s="3" t="s">
+        <v>401</v>
+      </c>
+      <c r="W5" s="3"/>
+      <c r="X5" s="3"/>
+      <c r="Y5" s="3"/>
+      <c r="Z5" s="3"/>
+      <c r="AA5" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="AB5" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="AC5" s="3"/>
+      <c r="AD5" s="3"/>
+      <c r="AE5" s="3"/>
+      <c r="AF5" s="3"/>
+      <c r="AG5" s="3"/>
+      <c r="AH5" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="AI5" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="AJ5" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="AK5" s="3"/>
+      <c r="AL5" s="3"/>
+      <c r="AM5" s="3"/>
+      <c r="AN5" s="3"/>
+    </row>
+    <row r="6" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="9"/>
+      <c r="B6" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="N6" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="O6" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="P6" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="Q6" s="3"/>
+      <c r="R6" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="S6" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="T6" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="U6" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="V6" s="3" t="s">
+        <v>402</v>
+      </c>
+      <c r="W6" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="X6" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="Y6" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="Z6" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="AA6" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="AB6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="AC6" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="AD6" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="AE6" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="AF6" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="AG6" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="AH6" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="AI6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="AJ6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="AK6" s="3"/>
+      <c r="AL6" s="3"/>
+      <c r="AM6" s="3"/>
+      <c r="AN6" s="3"/>
+    </row>
+    <row r="7" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="10"/>
+      <c r="B7" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="L7" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="M7" s="3" t="s">
+        <v>169</v>
+      </c>
+      <c r="N7" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="O7" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="P7" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q7" s="3"/>
+      <c r="R7" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="S7" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="T7" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="U7" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="V7" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="W7" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="X7" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="Y7" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="Z7" s="3"/>
+      <c r="AA7" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="AB7" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="AC7" s="3"/>
+      <c r="AD7" s="3"/>
+      <c r="AE7" s="3"/>
+      <c r="AF7" s="3"/>
+      <c r="AG7" s="3"/>
+      <c r="AH7" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="AI7" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="AJ7" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="AK7" s="3"/>
+      <c r="AL7" s="3"/>
+      <c r="AM7" s="3"/>
+      <c r="AN7" s="3"/>
+    </row>
+    <row r="8" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="11"/>
+      <c r="B8" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3" t="s">
+        <v>182</v>
+      </c>
+      <c r="J8" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="K8" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="M8" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="N8" s="3" t="s">
+        <v>186</v>
+      </c>
+      <c r="O8" s="3" t="s">
+        <v>187</v>
+      </c>
+      <c r="P8" s="3" t="s">
+        <v>188</v>
+      </c>
+      <c r="Q8" s="3" t="s">
+        <v>189</v>
+      </c>
+      <c r="R8" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="S8" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="T8" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="U8" s="3" t="s">
+        <v>191</v>
+      </c>
+      <c r="V8" s="3" t="s">
+        <v>404</v>
+      </c>
+      <c r="W8" s="3"/>
+      <c r="X8" s="3"/>
+      <c r="Y8" s="3"/>
+      <c r="Z8" s="3"/>
+      <c r="AA8" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="AB8" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="AC8" s="3"/>
+      <c r="AD8" s="3"/>
+      <c r="AE8" s="3"/>
+      <c r="AF8" s="3"/>
+      <c r="AG8" s="3"/>
+      <c r="AH8" s="3" t="s">
+        <v>192</v>
+      </c>
+      <c r="AI8" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="AJ8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="AK8" s="3"/>
+      <c r="AL8" s="3"/>
+      <c r="AM8" s="3"/>
+      <c r="AN8" s="3"/>
+    </row>
+    <row r="9" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="12"/>
+      <c r="B9" s="3" t="s">
+        <v>210</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="J9" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="K9" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="L9" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="M9" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="N9" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="O9" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="P9" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="Q9" s="3"/>
+      <c r="R9" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="S9" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="T9" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="U9" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="V9" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="W9" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="X9" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="Y9" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="Z9" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="AA9" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="AB9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="AC9" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="AD9" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="AE9" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="AF9" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="AG9" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="AH9" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="AI9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="AJ9" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="AK9" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="AL9" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="AM9" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="AN9" s="3" t="s">
+        <v>230</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="AH4" r:id="rId1" xr:uid="{939D6BFA-866E-47FE-A167-60E9B33C4530}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -3707,8 +3701,8 @@
       </c>
     </row>
     <row r="2" spans="1:33" x14ac:dyDescent="0.35">
-      <c r="A2" s="28" t="s">
-        <v>391</v>
+      <c r="A2" s="30" t="s">
+        <v>6</v>
       </c>
       <c r="B2" t="s" s="0">
         <v>7</v>
@@ -3805,7 +3799,7 @@
       </c>
     </row>
     <row r="3" spans="1:33" x14ac:dyDescent="0.35">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="31" t="s">
         <v>6</v>
       </c>
       <c r="B3" t="s" s="0">
@@ -3882,7 +3876,7 @@
       </c>
     </row>
     <row r="4" spans="1:33" x14ac:dyDescent="0.35">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="32" t="s">
         <v>6</v>
       </c>
       <c r="B4" t="s" s="0">
@@ -3959,7 +3953,7 @@
       </c>
     </row>
     <row r="5" spans="1:33" x14ac:dyDescent="0.35">
-      <c r="A5" s="8" t="s">
+      <c r="A5" s="33" t="s">
         <v>6</v>
       </c>
       <c r="B5" t="s" s="0">
@@ -4057,7 +4051,7 @@
       </c>
     </row>
     <row r="6" spans="1:33" x14ac:dyDescent="0.35">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="34" t="s">
         <v>6</v>
       </c>
       <c r="B6" t="s" s="0">
@@ -4134,7 +4128,7 @@
       </c>
     </row>
     <row r="7" spans="1:33" x14ac:dyDescent="0.35">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="35" t="s">
         <v>6</v>
       </c>
       <c r="B7" t="s" s="0">
@@ -4177,7 +4171,7 @@
         <v>100</v>
       </c>
       <c r="P7" t="s" s="0">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="Q7" t="s" s="0">
         <v>299</v>
@@ -4211,7 +4205,7 @@
       </c>
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.35">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="36" t="s">
         <v>6</v>
       </c>
       <c r="B8" t="s" s="0">
@@ -4288,7 +4282,7 @@
       </c>
     </row>
     <row r="9" spans="1:33" x14ac:dyDescent="0.35">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="37" t="s">
         <v>6</v>
       </c>
       <c r="B9" t="s" s="0">
@@ -4395,14 +4389,13 @@
   <dimension ref="A1:U2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" bestFit="true" customWidth="true" width="5.90625"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" width="6.90625"/>
+    <col min="1" max="2" bestFit="true" customWidth="true" width="5.90625"/>
     <col min="3" max="3" bestFit="true" customWidth="true" width="11.81640625"/>
     <col min="4" max="4" bestFit="true" customWidth="true" width="10.81640625"/>
-    <col min="5" max="5" bestFit="true" customWidth="true" width="23.6328125"/>
+    <col min="5" max="5" bestFit="true" customWidth="true" width="7.90625"/>
     <col min="6" max="6" bestFit="true" customWidth="true" width="9.7265625"/>
     <col min="7" max="7" bestFit="true" customWidth="true" width="11.36328125"/>
-    <col min="8" max="8" bestFit="true" customWidth="true" width="12.6328125"/>
+    <col min="8" max="8" bestFit="true" customWidth="true" width="9.0"/>
     <col min="9" max="9" bestFit="true" customWidth="true" width="3.81640625"/>
     <col min="10" max="10" bestFit="true" customWidth="true" width="8.36328125"/>
     <col min="11" max="11" bestFit="true" customWidth="true" width="7.7265625"/>
@@ -4410,6 +4403,12 @@
     <col min="13" max="13" bestFit="true" customWidth="true" width="10.54296875"/>
     <col min="14" max="14" bestFit="true" customWidth="true" width="9.81640625"/>
     <col min="15" max="15" bestFit="true" customWidth="true" width="7.36328125"/>
+    <col min="16" max="16" bestFit="true" customWidth="true" width="10.81640625"/>
+    <col min="17" max="17" bestFit="true" customWidth="true" width="8.81640625"/>
+    <col min="18" max="18" bestFit="true" customWidth="true" width="7.81640625"/>
+    <col min="19" max="19" bestFit="true" customWidth="true" width="12.90625"/>
+    <col min="20" max="20" bestFit="true" customWidth="true" width="11.1796875"/>
+    <col min="21" max="21" bestFit="true" customWidth="true" width="10.54296875"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="17" customHeight="1" x14ac:dyDescent="0.35">
@@ -4456,30 +4455,30 @@
         <v>338</v>
       </c>
       <c r="O1" t="s" s="0">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="P1" t="s" s="0">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="Q1" t="s" s="0">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="R1" t="s" s="0">
-        <v>396</v>
+        <v>392</v>
       </c>
       <c r="S1" t="s" s="0">
         <v>81</v>
       </c>
       <c r="T1" t="s" s="0">
-        <v>399</v>
+        <v>395</v>
       </c>
       <c r="U1" t="s" s="0">
-        <v>400</v>
+        <v>396</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A2" s="31" t="s">
-        <v>391</v>
+      <c r="A2" s="42" t="s">
+        <v>6</v>
       </c>
       <c r="B2" t="s" s="0">
         <v>7</v>
@@ -4491,7 +4490,7 @@
         <v>9965331986</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>406</v>
+        <v>385</v>
       </c>
       <c r="H2" t="s" s="0">
         <v>164</v>
@@ -4503,22 +4502,22 @@
         <v>339</v>
       </c>
       <c r="P2" t="s" s="0">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="Q2" t="s" s="0">
+        <v>393</v>
+      </c>
+      <c r="R2" t="s" s="0">
+        <v>394</v>
+      </c>
+      <c r="S2" s="6" t="s">
         <v>397</v>
       </c>
-      <c r="R2" t="s" s="0">
-        <v>398</v>
-      </c>
-      <c r="S2" s="29" t="s">
-        <v>401</v>
-      </c>
       <c r="T2" t="s" s="0">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="U2" t="s" s="0">
-        <v>397</v>
+        <v>393</v>
       </c>
     </row>
   </sheetData>
@@ -4652,48 +4651,48 @@
         <v>362</v>
       </c>
       <c r="AB1" t="s" s="0">
+        <v>377</v>
+      </c>
+      <c r="AC1" t="s" s="0">
         <v>378</v>
       </c>
-      <c r="AC1" t="s" s="0">
+      <c r="AD1" t="s" s="0">
         <v>379</v>
       </c>
-      <c r="AD1" t="s" s="0">
+      <c r="AE1" t="s" s="0">
+        <v>382</v>
+      </c>
+      <c r="AF1" t="s" s="0">
         <v>380</v>
       </c>
-      <c r="AE1" t="s" s="0">
-        <v>383</v>
-      </c>
-      <c r="AF1" t="s" s="0">
-        <v>381</v>
-      </c>
       <c r="AG1" t="s" s="0">
-        <v>385</v>
+        <v>384</v>
       </c>
       <c r="AH1" t="s" s="0">
-        <v>393</v>
+        <v>389</v>
       </c>
       <c r="AI1" t="s" s="0">
-        <v>394</v>
+        <v>390</v>
       </c>
       <c r="AJ1" t="s" s="0">
-        <v>395</v>
+        <v>391</v>
       </c>
       <c r="AK1" t="s" s="0">
-        <v>396</v>
+        <v>392</v>
       </c>
       <c r="AL1" t="s" s="0">
         <v>81</v>
       </c>
       <c r="AM1" t="s" s="0">
-        <v>399</v>
+        <v>395</v>
       </c>
       <c r="AN1" t="s" s="0">
-        <v>400</v>
+        <v>396</v>
       </c>
     </row>
     <row r="2" spans="1:40" x14ac:dyDescent="0.35">
-      <c r="A2" s="30" t="s">
-        <v>391</v>
+      <c r="A2" s="43" t="s">
+        <v>6</v>
       </c>
       <c r="B2" t="s" s="0">
         <v>363</v>
@@ -4702,7 +4701,7 @@
         <v>9965331986</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>405</v>
+        <v>400</v>
       </c>
       <c r="E2" t="s" s="0">
         <v>368</v>
@@ -4756,7 +4755,7 @@
         <v>46167</v>
       </c>
       <c r="X2" t="s" s="0">
-        <v>403</v>
+        <v>398</v>
       </c>
       <c r="Y2" s="0">
         <v>93209</v>
@@ -4780,28 +4779,31 @@
         <v>0</v>
       </c>
       <c r="AF2" t="s" s="0">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="AG2" s="0">
         <v>1000</v>
       </c>
+      <c r="AH2" t="s" s="0">
+        <v>428</v>
+      </c>
       <c r="AI2" t="s" s="0">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="AJ2" t="s" s="0">
+        <v>393</v>
+      </c>
+      <c r="AK2" t="s" s="0">
+        <v>394</v>
+      </c>
+      <c r="AL2" s="6" t="s">
         <v>397</v>
       </c>
-      <c r="AK2" t="s" s="0">
-        <v>398</v>
-      </c>
-      <c r="AL2" s="29" t="s">
-        <v>401</v>
-      </c>
       <c r="AM2" t="s" s="0">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="AN2" t="s" s="0">
-        <v>397</v>
+        <v>393</v>
       </c>
     </row>
     <row r="5" spans="1:40" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Break sleep added for close
</commit_message>
<xml_diff>
--- a/kalarakal_updated.xlsx
+++ b/kalarakal_updated.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chella\eclipse-workspace\mavenCrm\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5275A366-2466-43E4-A045-853496D17BA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EAFE198-AD86-4D04-BA4D-E550694387B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Master" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="801" uniqueCount="430">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="807" uniqueCount="429">
   <si>
     <t>Status</t>
   </si>
@@ -1231,9 +1231,6 @@
     <t>XYZPC9999K</t>
   </si>
   <si>
-    <t>DG-not allocated</t>
-  </si>
-  <si>
     <t>Ukkadam</t>
   </si>
   <si>
@@ -1279,46 +1276,46 @@
     <t>tirupur</t>
   </si>
   <si>
-    <t>2 Pass 0 Fail</t>
-  </si>
-  <si>
-    <t>207 Sec</t>
-  </si>
-  <si>
-    <t>25 Sec</t>
-  </si>
-  <si>
-    <t>26 Sec</t>
-  </si>
-  <si>
-    <t>22 Sec</t>
-  </si>
-  <si>
-    <t>200 Sec</t>
+    <t>1 Pass 0 Fail</t>
+  </si>
+  <si>
+    <t>26-DG-38</t>
+  </si>
+  <si>
+    <t>Amount To Weight Scheme</t>
+  </si>
+  <si>
+    <t>TimeTaken</t>
+  </si>
+  <si>
+    <t>9 Sec</t>
+  </si>
+  <si>
+    <t>21 Sec</t>
+  </si>
+  <si>
+    <t>24 Sec</t>
+  </si>
+  <si>
+    <t>19 Sec</t>
+  </si>
+  <si>
+    <t>292 Sec</t>
+  </si>
+  <si>
+    <t>134 Sec</t>
+  </si>
+  <si>
+    <t>23 Sec</t>
   </si>
   <si>
     <t>14 Sec</t>
   </si>
   <si>
-    <t>1 Pass 0 Fail</t>
-  </si>
-  <si>
-    <t>34 Sec</t>
-  </si>
-  <si>
-    <t>19 Sec</t>
-  </si>
-  <si>
-    <t>12 Sec</t>
-  </si>
-  <si>
-    <t>36 Sec</t>
-  </si>
-  <si>
-    <t>26-DG-38</t>
-  </si>
-  <si>
-    <t>66 Sec</t>
+    <t>10 Sec</t>
+  </si>
+  <si>
+    <t>17 Sec</t>
   </si>
 </sst>
 </file>
@@ -1326,7 +1323,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="0"/>
-  <fonts count="41" x14ac:knownFonts="1">
+  <fonts count="40" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1347,6 +1344,18 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color indexed="17"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color indexed="10"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <b/>
@@ -1547,18 +1556,6 @@
       <name val="Calibri"/>
     </font>
     <font>
-      <b/>
-      <sz val="11"/>
-      <color indexed="17"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color indexed="10"/>
-      <name val="Calibri"/>
-    </font>
-    <font>
       <name val="Calibri"/>
       <sz val="11.0"/>
       <b val="true"/>
@@ -1568,13 +1565,7 @@
       <name val="Calibri"/>
       <sz val="11.0"/>
       <b val="true"/>
-      <color indexed="17"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-      <color indexed="17"/>
+      <color indexed="10"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1598,7 +1589,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="44">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
@@ -1644,7 +1635,6 @@
     <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="38" fillId="0" borderId="0" xfId="0" applyFont="true"/>
     <xf numFmtId="0" fontId="39" fillId="0" borderId="0" xfId="0" applyFont="true"/>
-    <xf numFmtId="0" fontId="40" fillId="0" borderId="0" xfId="0" applyFont="true"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1932,7 +1922,7 @@
     <col min="1" max="1" bestFit="true" customWidth="true" width="12.7265625"/>
     <col min="2" max="2" bestFit="true" customWidth="true" width="7.81640625"/>
     <col min="3" max="3" bestFit="true" customWidth="true" width="13.90625"/>
-    <col min="4" max="4" bestFit="true" customWidth="true" width="5.0"/>
+    <col min="4" max="4" bestFit="true" customWidth="true" width="9.90625"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
@@ -1945,6 +1935,9 @@
       <c r="C1" t="s" s="0">
         <v>22</v>
       </c>
+      <c r="D1" t="s" s="0">
+        <v>418</v>
+      </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A2" t="s" s="0">
@@ -1957,7 +1950,7 @@
         <v>387</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>426</v>
+        <v>427</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
@@ -1971,7 +1964,7 @@
         <v>373</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>418</v>
+        <v>420</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
@@ -1985,7 +1978,7 @@
         <v>373</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>419</v>
+        <v>421</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
@@ -1999,7 +1992,7 @@
         <v>373</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>420</v>
+        <v>422</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
@@ -2010,10 +2003,10 @@
         <v>9</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>416</v>
+        <v>376</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>417</v>
+        <v>423</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
@@ -2027,7 +2020,7 @@
         <v>376</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>421</v>
+        <v>424</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
@@ -2035,13 +2028,13 @@
         <v>27</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="C8" t="s" s="0">
-        <v>423</v>
+        <v>415</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>427</v>
+        <v>425</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
@@ -2052,10 +2045,10 @@
         <v>12</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>423</v>
+        <v>387</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
   </sheetData>
@@ -2185,7 +2178,7 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="8" t="s">
         <v>6</v>
       </c>
       <c r="B2" t="s" s="0">
@@ -2202,7 +2195,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="9" t="s">
         <v>6</v>
       </c>
       <c r="B3" t="s" s="0">
@@ -2222,7 +2215,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="10" t="s">
         <v>6</v>
       </c>
       <c r="B4" t="s" s="0">
@@ -2239,7 +2232,7 @@
       </c>
     </row>
     <row r="5" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="18" t="s">
+      <c r="A5" s="11" t="s">
         <v>6</v>
       </c>
       <c r="B5" t="s" s="0">
@@ -2259,7 +2252,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="14" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="12" t="s">
         <v>6</v>
       </c>
       <c r="B6" t="s" s="0">
@@ -2312,7 +2305,7 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="13" t="s">
         <v>6</v>
       </c>
       <c r="B2" t="s" s="0">
@@ -2329,7 +2322,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="14" t="s">
         <v>6</v>
       </c>
       <c r="B3" t="s" s="0">
@@ -2349,7 +2342,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="15" t="s">
         <v>6</v>
       </c>
       <c r="B4" t="s" s="0">
@@ -2366,7 +2359,7 @@
       </c>
     </row>
     <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="23" t="s">
+      <c r="A5" s="16" t="s">
         <v>6</v>
       </c>
       <c r="B5" t="s" s="0">
@@ -2386,7 +2379,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="17" t="s">
         <v>6</v>
       </c>
       <c r="B6" t="s" s="0">
@@ -2439,7 +2432,7 @@
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="18" t="s">
         <v>6</v>
       </c>
       <c r="B2" t="s" s="0">
@@ -2456,7 +2449,7 @@
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="26" t="s">
+      <c r="A3" s="19" t="s">
         <v>6</v>
       </c>
       <c r="B3" t="s" s="0">
@@ -2476,7 +2469,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" s="27" t="s">
+      <c r="A4" s="20" t="s">
         <v>6</v>
       </c>
       <c r="B4" t="s" s="0">
@@ -2493,7 +2486,7 @@
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="21" t="s">
         <v>6</v>
       </c>
       <c r="B5" t="s" s="0">
@@ -2513,7 +2506,7 @@
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A6" s="29" t="s">
+      <c r="A6" s="22" t="s">
         <v>6</v>
       </c>
       <c r="B6" t="s" s="0">
@@ -2702,20 +2695,22 @@
         <v>86</v>
       </c>
       <c r="AO1" t="s" s="0">
+        <v>407</v>
+      </c>
+      <c r="AP1" t="s" s="0">
         <v>408</v>
       </c>
-      <c r="AP1" t="s" s="0">
+      <c r="AQ1" t="s" s="0">
         <v>409</v>
       </c>
-      <c r="AQ1" t="s" s="0">
+      <c r="AR1" t="s" s="0">
         <v>410</v>
       </c>
-      <c r="AR1" t="s" s="0">
-        <v>411</v>
-      </c>
     </row>
     <row r="2" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="13"/>
+      <c r="A2" s="23" t="s">
+        <v>6</v>
+      </c>
       <c r="B2" s="3" t="s">
         <v>7</v>
       </c>
@@ -2773,7 +2768,7 @@
         <v>151</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
       <c r="W2" s="3" t="s">
         <v>152</v>
@@ -2830,14 +2825,16 @@
         <v>162</v>
       </c>
       <c r="AP2" t="s" s="0">
-        <v>413</v>
+        <v>412</v>
       </c>
       <c r="AR2" t="s" s="0">
         <v>393</v>
       </c>
     </row>
     <row r="3" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="14"/>
+      <c r="A3" s="24" t="s">
+        <v>6</v>
+      </c>
       <c r="B3" s="3" t="s">
         <v>10</v>
       </c>
@@ -2893,7 +2890,7 @@
         <v>204</v>
       </c>
       <c r="V3" s="3" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
       <c r="W3" s="3" t="s">
         <v>102</v>
@@ -2940,14 +2937,16 @@
       <c r="AM3" s="3"/>
       <c r="AN3" s="3"/>
       <c r="AQ3" t="s" s="0">
-        <v>414</v>
+        <v>413</v>
       </c>
       <c r="AR3" t="s" s="0">
         <v>393</v>
       </c>
     </row>
     <row r="4" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="7"/>
+      <c r="A4" s="25" t="s">
+        <v>6</v>
+      </c>
       <c r="B4" s="3" t="s">
         <v>14</v>
       </c>
@@ -3039,7 +3038,7 @@
         <v>98</v>
       </c>
       <c r="AH4" s="1" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
       <c r="AI4" s="3" t="s">
         <v>9</v>
@@ -3052,14 +3051,16 @@
       <c r="AM4" s="3"/>
       <c r="AN4" s="3"/>
       <c r="AO4" t="s" s="0">
-        <v>412</v>
+        <v>411</v>
       </c>
       <c r="AR4" t="s" s="0">
         <v>393</v>
       </c>
     </row>
     <row r="5" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="8"/>
+      <c r="A5" s="26" t="s">
+        <v>6</v>
+      </c>
       <c r="B5" s="3" t="s">
         <v>16</v>
       </c>
@@ -3117,7 +3118,7 @@
         <v>119</v>
       </c>
       <c r="V5" s="3" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="W5" s="3"/>
       <c r="X5" s="3"/>
@@ -3149,7 +3150,9 @@
       <c r="AN5" s="3"/>
     </row>
     <row r="6" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="9"/>
+      <c r="A6" s="27" t="s">
+        <v>6</v>
+      </c>
       <c r="B6" s="3" t="s">
         <v>18</v>
       </c>
@@ -3205,7 +3208,7 @@
         <v>132</v>
       </c>
       <c r="V6" s="3" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
       <c r="W6" s="3" t="s">
         <v>102</v>
@@ -3255,7 +3258,9 @@
       <c r="AN6" s="3"/>
     </row>
     <row r="7" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="10"/>
+      <c r="A7" s="28" t="s">
+        <v>6</v>
+      </c>
       <c r="B7" s="3" t="s">
         <v>18</v>
       </c>
@@ -3311,7 +3316,7 @@
         <v>174</v>
       </c>
       <c r="V7" s="3" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="W7" s="3" t="s">
         <v>175</v>
@@ -3349,7 +3354,9 @@
       <c r="AN7" s="3"/>
     </row>
     <row r="8" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="11"/>
+      <c r="A8" s="29" t="s">
+        <v>6</v>
+      </c>
       <c r="B8" s="3" t="s">
         <v>179</v>
       </c>
@@ -3407,7 +3414,7 @@
         <v>191</v>
       </c>
       <c r="V8" s="3" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="W8" s="3"/>
       <c r="X8" s="3"/>
@@ -3439,7 +3446,9 @@
       <c r="AN8" s="3"/>
     </row>
     <row r="9" spans="1:44" ht="17" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="12"/>
+      <c r="A9" s="30" t="s">
+        <v>6</v>
+      </c>
       <c r="B9" s="3" t="s">
         <v>210</v>
       </c>
@@ -3495,7 +3504,7 @@
         <v>221</v>
       </c>
       <c r="V9" s="3" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
       <c r="W9" s="3" t="s">
         <v>102</v>
@@ -3701,7 +3710,7 @@
       </c>
     </row>
     <row r="2" spans="1:33" x14ac:dyDescent="0.35">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="31" t="s">
         <v>6</v>
       </c>
       <c r="B2" t="s" s="0">
@@ -3799,7 +3808,7 @@
       </c>
     </row>
     <row r="3" spans="1:33" x14ac:dyDescent="0.35">
-      <c r="A3" s="31" t="s">
+      <c r="A3" s="32" t="s">
         <v>6</v>
       </c>
       <c r="B3" t="s" s="0">
@@ -3876,7 +3885,7 @@
       </c>
     </row>
     <row r="4" spans="1:33" x14ac:dyDescent="0.35">
-      <c r="A4" s="32" t="s">
+      <c r="A4" s="33" t="s">
         <v>6</v>
       </c>
       <c r="B4" t="s" s="0">
@@ -3953,7 +3962,7 @@
       </c>
     </row>
     <row r="5" spans="1:33" x14ac:dyDescent="0.35">
-      <c r="A5" s="33" t="s">
+      <c r="A5" s="34" t="s">
         <v>6</v>
       </c>
       <c r="B5" t="s" s="0">
@@ -4051,7 +4060,7 @@
       </c>
     </row>
     <row r="6" spans="1:33" x14ac:dyDescent="0.35">
-      <c r="A6" s="34" t="s">
+      <c r="A6" s="35" t="s">
         <v>6</v>
       </c>
       <c r="B6" t="s" s="0">
@@ -4128,7 +4137,7 @@
       </c>
     </row>
     <row r="7" spans="1:33" x14ac:dyDescent="0.35">
-      <c r="A7" s="35" t="s">
+      <c r="A7" s="36" t="s">
         <v>6</v>
       </c>
       <c r="B7" t="s" s="0">
@@ -4205,7 +4214,7 @@
       </c>
     </row>
     <row r="8" spans="1:33" x14ac:dyDescent="0.35">
-      <c r="A8" s="36" t="s">
+      <c r="A8" s="37" t="s">
         <v>6</v>
       </c>
       <c r="B8" t="s" s="0">
@@ -4282,7 +4291,7 @@
       </c>
     </row>
     <row r="9" spans="1:33" x14ac:dyDescent="0.35">
-      <c r="A9" s="37" t="s">
+      <c r="A9" s="38" t="s">
         <v>6</v>
       </c>
       <c r="B9" t="s" s="0">
@@ -4477,7 +4486,7 @@
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.35">
-      <c r="A2" s="42" t="s">
+      <c r="A2" s="39" t="s">
         <v>6</v>
       </c>
       <c r="B2" t="s" s="0">
@@ -4490,7 +4499,7 @@
         <v>9965331986</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>385</v>
+        <v>417</v>
       </c>
       <c r="H2" t="s" s="0">
         <v>164</v>
@@ -4500,6 +4509,9 @@
       </c>
       <c r="N2" t="s" s="0">
         <v>339</v>
+      </c>
+      <c r="O2" s="0">
+        <v>1000</v>
       </c>
       <c r="P2" t="s" s="0">
         <v>399</v>
@@ -4691,8 +4703,8 @@
       </c>
     </row>
     <row r="2" spans="1:40" x14ac:dyDescent="0.35">
-      <c r="A2" s="43" t="s">
-        <v>6</v>
+      <c r="A2" s="42" t="s">
+        <v>388</v>
       </c>
       <c r="B2" t="s" s="0">
         <v>363</v>
@@ -4701,7 +4713,7 @@
         <v>9965331986</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>400</v>
+        <v>416</v>
       </c>
       <c r="E2" t="s" s="0">
         <v>368</v>
@@ -4785,7 +4797,7 @@
         <v>1000</v>
       </c>
       <c r="AH2" t="s" s="0">
-        <v>428</v>
+        <v>416</v>
       </c>
       <c r="AI2" t="s" s="0">
         <v>399</v>

</xml_diff>